<commit_message>
Update Bant Boys results; add 2026 master
Refresh Bant Boys standings and related race data. Updated placements, points and rider entries across data/division_results.json, data/race_comparison.json, data/results.json, data/school_results.json and data/team_results.json to reflect corrected R1/R2 results and recalculated totals. Added results_2026_master.xlsx and its temporary ~$ file.
</commit_message>
<xml_diff>
--- a/results_2026_master.xlsx
+++ b/results_2026_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\19247\Documents\codemathbike\codemathbike_bike\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{962FCAA7-C42B-462D-B51C-C29237F60E3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2F84A13-8917-4216-9119-36C70B822CC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{E4CCCC36-747C-4C6A-A938-400850181E6F}"/>
   </bookViews>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2304" uniqueCount="419">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2323" uniqueCount="419">
   <si>
     <t>Divisions</t>
   </si>
@@ -1438,7 +1438,14 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="44">
+  <dxfs count="45">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1804,7 +1811,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B67B0C24-496D-4362-8989-27568D29525A}" name="tbl_points" displayName="tbl_points" ref="E1:F60" totalsRowShown="0" headerRowDxfId="43">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B67B0C24-496D-4362-8989-27568D29525A}" name="tbl_points" displayName="tbl_points" ref="E1:F60" totalsRowShown="0" headerRowDxfId="44">
   <autoFilter ref="E1:F60" xr:uid="{B67B0C24-496D-4362-8989-27568D29525A}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{26FEA31D-C1DD-4A82-A0F0-29F4BFEAA9BF}" name="Place"/>
@@ -1815,7 +1822,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{4732A653-9976-4BC3-B1BB-3377C0BE5451}" name="tbl_individual" displayName="tbl_individual" ref="A1:S353" totalsRowShown="0" headerRowDxfId="42">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{4732A653-9976-4BC3-B1BB-3377C0BE5451}" name="tbl_individual" displayName="tbl_individual" ref="A1:S353" totalsRowShown="0" headerRowDxfId="43">
   <autoFilter ref="A1:S353" xr:uid="{4732A653-9976-4BC3-B1BB-3377C0BE5451}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S353">
     <sortCondition ref="S1:S353"/>
@@ -1824,38 +1831,38 @@
     <tableColumn id="1" xr3:uid="{DD0C8BFC-D933-4D84-A252-784AFB91D5D2}" name="Student Name"/>
     <tableColumn id="2" xr3:uid="{50DB066B-1368-4510-AE03-F035E82A9C80}" name="School"/>
     <tableColumn id="3" xr3:uid="{7521EB7C-E51A-4930-A4D2-608C8D120FA9}" name="Division"/>
-    <tableColumn id="4" xr3:uid="{95AF9BEA-E11E-4C3A-98F5-4C1CA2AE9261}" name="Plate #" dataDxfId="41"/>
-    <tableColumn id="5" xr3:uid="{C4BC7103-4C35-4FC3-8F18-8455C41D4783}" name="R1 Place" dataDxfId="40"/>
-    <tableColumn id="6" xr3:uid="{F003CE6A-1709-47C7-A52B-4E78A06B55BC}" name="R1 Pts" dataDxfId="39">
+    <tableColumn id="4" xr3:uid="{95AF9BEA-E11E-4C3A-98F5-4C1CA2AE9261}" name="Plate #" dataDxfId="42"/>
+    <tableColumn id="5" xr3:uid="{C4BC7103-4C35-4FC3-8F18-8455C41D4783}" name="R1 Place" dataDxfId="41"/>
+    <tableColumn id="6" xr3:uid="{F003CE6A-1709-47C7-A52B-4E78A06B55BC}" name="R1 Pts" dataDxfId="40">
       <calculatedColumnFormula>IF(E2="","",IF(E2="DNS",0,IF(E2="DQ",0,IF(E2="DNF",1,IF(AND(ISNUMBER(E2),E2&gt;59),1,_xlfn.XLOOKUP(E2,tbl_points[Place],tbl_points[Points],""))))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00AA5EEC-F524-4B3A-8D3D-DD590338CBF4}" name="R2 Place" dataDxfId="38"/>
-    <tableColumn id="8" xr3:uid="{D5BD0204-BF0C-4CD7-84CF-355F4C709D84}" name="R2 Pts" dataDxfId="37">
+    <tableColumn id="7" xr3:uid="{00AA5EEC-F524-4B3A-8D3D-DD590338CBF4}" name="R2 Place" dataDxfId="39"/>
+    <tableColumn id="8" xr3:uid="{D5BD0204-BF0C-4CD7-84CF-355F4C709D84}" name="R2 Pts" dataDxfId="38">
       <calculatedColumnFormula>IF(G2="","",IF(G2="DNS",0,IF(G2="DQ",0,IF(G2="DNF",1,IF(AND(ISNUMBER(G2),G2&gt;59),1,_xlfn.XLOOKUP(G2,tbl_points[Place],tbl_points[Points],""))))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{AAA1602A-3E76-4D80-A749-C082B0EEE022}" name="R3 Place" dataDxfId="36"/>
-    <tableColumn id="10" xr3:uid="{129B956B-A68A-4A58-B03A-5E88F63F4109}" name="R3 Pts" dataDxfId="35">
+    <tableColumn id="9" xr3:uid="{AAA1602A-3E76-4D80-A749-C082B0EEE022}" name="R3 Place" dataDxfId="37"/>
+    <tableColumn id="10" xr3:uid="{129B956B-A68A-4A58-B03A-5E88F63F4109}" name="R3 Pts" dataDxfId="36">
       <calculatedColumnFormula>IF(I2="","",IF(I2="DNS",0,IF(I2="DQ",0,IF(I2="DNF",1,IF(AND(ISNUMBER(I2),I2&gt;59),1,_xlfn.XLOOKUP(I2,tbl_points[Place],tbl_points[Points],""))))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{58CEE06C-D397-4C16-AFDA-197232873DB1}" name="R4 Place" dataDxfId="34"/>
-    <tableColumn id="12" xr3:uid="{8F6D618C-1190-4F5C-A449-77BB8AFE782C}" name="R4 Pts" dataDxfId="33">
+    <tableColumn id="11" xr3:uid="{58CEE06C-D397-4C16-AFDA-197232873DB1}" name="R4 Place" dataDxfId="35"/>
+    <tableColumn id="12" xr3:uid="{8F6D618C-1190-4F5C-A449-77BB8AFE782C}" name="R4 Pts" dataDxfId="34">
       <calculatedColumnFormula>IF(K2="","",IF(K2="DNS",0,IF(K2="DQ",0,IF(K2="DNF",1,IF(AND(ISNUMBER(K2),K2&gt;59),1,_xlfn.XLOOKUP(K2,tbl_points[Place],tbl_points[Points],""))))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{09134E3A-40B6-4480-BF56-619415F1546B}" name="R5 Place" dataDxfId="32"/>
-    <tableColumn id="14" xr3:uid="{0630E922-C5AC-4446-B509-709B7EECF31A}" name="R5 Pts" dataDxfId="31">
+    <tableColumn id="13" xr3:uid="{09134E3A-40B6-4480-BF56-619415F1546B}" name="R5 Place" dataDxfId="33"/>
+    <tableColumn id="14" xr3:uid="{0630E922-C5AC-4446-B509-709B7EECF31A}" name="R5 Pts" dataDxfId="32">
       <calculatedColumnFormula>IF(M2="","",IF(M2="DNS",0,IF(M2="DQ",0,IF(M2="DNF",1,IF(AND(ISNUMBER(M2),M2&gt;59),1,_xlfn.XLOOKUP(M2,tbl_points[Place],tbl_points[Points],""))))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{A3A3C6B1-EAC4-4CA1-B9F1-91AD4AED8E96}" name="R6 Place" dataDxfId="30"/>
-    <tableColumn id="16" xr3:uid="{183BA364-7ECF-4FCA-8D96-4CEAFE4D6897}" name="R6 Pts" dataDxfId="29">
+    <tableColumn id="15" xr3:uid="{A3A3C6B1-EAC4-4CA1-B9F1-91AD4AED8E96}" name="R6 Place" dataDxfId="31"/>
+    <tableColumn id="16" xr3:uid="{183BA364-7ECF-4FCA-8D96-4CEAFE4D6897}" name="R6 Pts" dataDxfId="30">
       <calculatedColumnFormula>IF(O2="","",IF(O2="DNS",0,IF(O2="DQ",0,IF(O2="DNF",1,IF(AND(ISNUMBER(O2),O2&gt;59),1,_xlfn.XLOOKUP(O2,tbl_points[Place],tbl_points[Points],""))))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{7E434874-15F0-4158-8350-07E2BFD885BE}" name="Total" dataDxfId="28">
+    <tableColumn id="17" xr3:uid="{7E434874-15F0-4158-8350-07E2BFD885BE}" name="Total" dataDxfId="29">
       <calculatedColumnFormula>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{86859925-B685-41CB-B33D-9607A1626666}" name="Lowest Score" dataDxfId="27">
+    <tableColumn id="18" xr3:uid="{86859925-B685-41CB-B33D-9607A1626666}" name="Lowest Score" dataDxfId="28">
       <calculatedColumnFormula>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{3B09C5B7-0CED-45E4-9DF3-6F0F3B8C89EE}" name="Top 5" dataDxfId="0">
+    <tableColumn id="19" xr3:uid="{3B09C5B7-0CED-45E4-9DF3-6F0F3B8C89EE}" name="Top 5" dataDxfId="1">
       <calculatedColumnFormula>tbl_individual[[#This Row],[Total]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1864,13 +1871,13 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{10951E40-9465-4D54-A308-3E2A245DA857}" name="enduro" displayName="enduro" ref="A1:E353" totalsRowShown="0" headerRowDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{10951E40-9465-4D54-A308-3E2A245DA857}" name="enduro" displayName="enduro" ref="A1:E353" totalsRowShown="0" headerRowDxfId="2">
   <autoFilter ref="A1:E353" xr:uid="{10951E40-9465-4D54-A308-3E2A245DA857}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F5B760F2-2C17-4991-A9D6-EED4261386D4}" name="Student Name"/>
     <tableColumn id="2" xr3:uid="{7CB5820D-3B26-4DA7-9C21-32B6A5DC2026}" name="School"/>
     <tableColumn id="3" xr3:uid="{9F55042D-35BF-4BB8-9118-1298A4D8E67F}" name="Division"/>
-    <tableColumn id="4" xr3:uid="{5F574A16-C593-44D6-BF33-5771DDE10346}" name="Plate #" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{5F574A16-C593-44D6-BF33-5771DDE10346}" name="Plate #" dataDxfId="3"/>
     <tableColumn id="5" xr3:uid="{76D035DA-EC5A-4955-8134-6D150CD5B699}" name="yes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1878,12 +1885,12 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{6FE32177-DBD8-4299-9E12-DE45C01CDFC1}" name="tbl_teampoints" displayName="tbl_teampoints" ref="A1:I47" totalsRowShown="0" headerRowDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{6FE32177-DBD8-4299-9E12-DE45C01CDFC1}" name="tbl_teampoints" displayName="tbl_teampoints" ref="A1:I47" totalsRowShown="0" headerRowDxfId="27">
   <autoFilter ref="A1:I47" xr:uid="{6FE32177-DBD8-4299-9E12-DE45C01CDFC1}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{E4DDB9C1-470A-4B63-B391-B74364B13A0B}" name="Division"/>
     <tableColumn id="2" xr3:uid="{C9B23502-0457-486C-96DF-CDE7023AF0B8}" name="School"/>
-    <tableColumn id="3" xr3:uid="{2FDC0DE4-1DEE-4FF2-90E4-1CEBC22D34E1}" name="Race 1" dataDxfId="25">
+    <tableColumn id="3" xr3:uid="{2FDC0DE4-1DEE-4FF2-90E4-1CEBC22D34E1}" name="Race 1" dataDxfId="26">
       <calculatedColumnFormula array="1">_xlfn.LET(
 _xlpm.teamDiv,tbl_teampoints[[#This Row],[Division]],
 _xlpm.teamSchool,tbl_teampoints[[#This Row],[School]],
@@ -1915,7 +1922,7 @@
 )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{B1A9F92E-C531-4F9B-9E61-4AF67269E504}" name="Race 2" dataDxfId="24">
+    <tableColumn id="4" xr3:uid="{B1A9F92E-C531-4F9B-9E61-4AF67269E504}" name="Race 2" dataDxfId="25">
       <calculatedColumnFormula array="1">_xlfn.LET(
 _xlpm.teamDiv,tbl_teampoints[[#This Row],[Division]],
 _xlpm.teamSchool,tbl_teampoints[[#This Row],[School]],
@@ -1947,7 +1954,7 @@
 )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{98622B84-034F-49A3-94EB-FE028D7330DC}" name="Race 3" dataDxfId="23">
+    <tableColumn id="5" xr3:uid="{98622B84-034F-49A3-94EB-FE028D7330DC}" name="Race 3" dataDxfId="24">
       <calculatedColumnFormula array="1">_xlfn.LET(
 _xlpm.teamDiv,tbl_teampoints[[#This Row],[Division]],
 _xlpm.teamSchool,tbl_teampoints[[#This Row],[School]],
@@ -1979,7 +1986,7 @@
 )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{E251564D-BEF9-4A06-B705-57876A4C364D}" name="Race 4" dataDxfId="22">
+    <tableColumn id="6" xr3:uid="{E251564D-BEF9-4A06-B705-57876A4C364D}" name="Race 4" dataDxfId="23">
       <calculatedColumnFormula array="1">_xlfn.LET(
 _xlpm.teamDiv,tbl_teampoints[[#This Row],[Division]],
 _xlpm.teamSchool,tbl_teampoints[[#This Row],[School]],
@@ -2011,7 +2018,7 @@
 )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{E38A2690-1CC8-45F7-9CAB-D28FDE2604B7}" name="Race 5" dataDxfId="21">
+    <tableColumn id="7" xr3:uid="{E38A2690-1CC8-45F7-9CAB-D28FDE2604B7}" name="Race 5" dataDxfId="22">
       <calculatedColumnFormula array="1">_xlfn.LET(
 _xlpm.teamDiv,tbl_teampoints[[#This Row],[Division]],
 _xlpm.teamSchool,tbl_teampoints[[#This Row],[School]],
@@ -2043,7 +2050,7 @@
 )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{51FAA391-8BE1-4ECE-A0AB-B5AB0C9BE2C5}" name="Race 6" dataDxfId="20">
+    <tableColumn id="8" xr3:uid="{51FAA391-8BE1-4ECE-A0AB-B5AB0C9BE2C5}" name="Race 6" dataDxfId="21">
       <calculatedColumnFormula array="1">_xlfn.LET(
 _xlpm.teamDiv,tbl_teampoints[[#This Row],[Division]],
 _xlpm.teamSchool,tbl_teampoints[[#This Row],[School]],
@@ -2075,7 +2082,7 @@
 )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{539A3327-6FEC-4B8A-A923-635DC3180909}" name="Total" dataDxfId="19">
+    <tableColumn id="9" xr3:uid="{539A3327-6FEC-4B8A-A923-635DC3180909}" name="Total" dataDxfId="20">
       <calculatedColumnFormula>SUM(tbl_teampoints[[#This Row],[Race 1]]:tbl_teampoints[[#This Row],[Race 6]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3105,9 +3112,12 @@
         <f>IF(E2="","",IF(E2="DNS",0,IF(E2="DQ",0,IF(E2="DNF",1,IF(AND(ISNUMBER(E2),E2&gt;59),1,_xlfn.XLOOKUP(E2,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>45</v>
       </c>
-      <c r="H2" s="3" t="str">
+      <c r="G2" s="3">
+        <v>25</v>
+      </c>
+      <c r="H2" s="3">
         <f>IF(G2="","",IF(G2="DNS",0,IF(G2="DQ",0,IF(G2="DNF",1,IF(AND(ISNUMBER(G2),G2&gt;59),1,_xlfn.XLOOKUP(G2,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>35</v>
       </c>
       <c r="J2" s="3" t="str">
         <f>IF(I2="","",IF(I2="DNS",0,IF(I2="DQ",0,IF(I2="DNF",1,IF(AND(ISNUMBER(I2),I2&gt;59),1,_xlfn.XLOOKUP(I2,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -3127,15 +3137,15 @@
       </c>
       <c r="Q2" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="R2" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="S2" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>45</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.4">
@@ -3158,9 +3168,12 @@
         <f>IF(E3="","",IF(E3="DNS",0,IF(E3="DQ",0,IF(E3="DNF",1,IF(AND(ISNUMBER(E3),E3&gt;59),1,_xlfn.XLOOKUP(E3,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>0</v>
       </c>
-      <c r="H3" s="3" t="str">
+      <c r="G3" s="3">
+        <v>1</v>
+      </c>
+      <c r="H3" s="3">
         <f>IF(G3="","",IF(G3="DNS",0,IF(G3="DQ",0,IF(G3="DNF",1,IF(AND(ISNUMBER(G3),G3&gt;59),1,_xlfn.XLOOKUP(G3,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>100</v>
       </c>
       <c r="J3" s="3" t="str">
         <f>IF(I3="","",IF(I3="DNS",0,IF(I3="DQ",0,IF(I3="DNF",1,IF(AND(ISNUMBER(I3),I3&gt;59),1,_xlfn.XLOOKUP(I3,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -3180,7 +3193,7 @@
       </c>
       <c r="Q3" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R3" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -3188,7 +3201,7 @@
       </c>
       <c r="S3" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.4">
@@ -3211,9 +3224,12 @@
         <f>IF(E4="","",IF(E4="DNS",0,IF(E4="DQ",0,IF(E4="DNF",1,IF(AND(ISNUMBER(E4),E4&gt;59),1,_xlfn.XLOOKUP(E4,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>95</v>
       </c>
-      <c r="H4" s="3" t="str">
+      <c r="G4" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="H4" s="3">
         <f>IF(G4="","",IF(G4="DNS",0,IF(G4="DQ",0,IF(G4="DNF",1,IF(AND(ISNUMBER(G4),G4&gt;59),1,_xlfn.XLOOKUP(G4,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J4" s="3" t="str">
         <f>IF(I4="","",IF(I4="DNS",0,IF(I4="DQ",0,IF(I4="DNF",1,IF(AND(ISNUMBER(I4),I4&gt;59),1,_xlfn.XLOOKUP(I4,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -3237,7 +3253,7 @@
       </c>
       <c r="R4" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="S4" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
@@ -3264,9 +3280,12 @@
         <f>IF(E5="","",IF(E5="DNS",0,IF(E5="DQ",0,IF(E5="DNF",1,IF(AND(ISNUMBER(E5),E5&gt;59),1,_xlfn.XLOOKUP(E5,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>85</v>
       </c>
-      <c r="H5" s="3" t="str">
+      <c r="G5" s="3">
+        <v>20</v>
+      </c>
+      <c r="H5" s="3">
         <f>IF(G5="","",IF(G5="DNS",0,IF(G5="DQ",0,IF(G5="DNF",1,IF(AND(ISNUMBER(G5),G5&gt;59),1,_xlfn.XLOOKUP(G5,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>40</v>
       </c>
       <c r="J5" s="3" t="str">
         <f>IF(I5="","",IF(I5="DNS",0,IF(I5="DQ",0,IF(I5="DNF",1,IF(AND(ISNUMBER(I5),I5&gt;59),1,_xlfn.XLOOKUP(I5,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -3286,15 +3305,15 @@
       </c>
       <c r="Q5" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>85</v>
+        <v>125</v>
       </c>
       <c r="R5" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>85</v>
+        <v>40</v>
       </c>
       <c r="S5" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>85</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.4">
@@ -3317,9 +3336,12 @@
         <f>IF(E6="","",IF(E6="DNS",0,IF(E6="DQ",0,IF(E6="DNF",1,IF(AND(ISNUMBER(E6),E6&gt;59),1,_xlfn.XLOOKUP(E6,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>42</v>
       </c>
-      <c r="H6" s="3" t="str">
+      <c r="G6" s="3">
+        <v>34</v>
+      </c>
+      <c r="H6" s="3">
         <f>IF(G6="","",IF(G6="DNS",0,IF(G6="DQ",0,IF(G6="DNF",1,IF(AND(ISNUMBER(G6),G6&gt;59),1,_xlfn.XLOOKUP(G6,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>26</v>
       </c>
       <c r="J6" s="3" t="str">
         <f>IF(I6="","",IF(I6="DNS",0,IF(I6="DQ",0,IF(I6="DNF",1,IF(AND(ISNUMBER(I6),I6&gt;59),1,_xlfn.XLOOKUP(I6,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -3339,15 +3361,15 @@
       </c>
       <c r="Q6" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>42</v>
+        <v>68</v>
       </c>
       <c r="R6" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="S6" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>42</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.4">
@@ -3370,9 +3392,12 @@
         <f>IF(E7="","",IF(E7="DNS",0,IF(E7="DQ",0,IF(E7="DNF",1,IF(AND(ISNUMBER(E7),E7&gt;59),1,_xlfn.XLOOKUP(E7,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>0</v>
       </c>
-      <c r="H7" s="3" t="str">
+      <c r="G7" s="3">
+        <v>16</v>
+      </c>
+      <c r="H7" s="3">
         <f>IF(G7="","",IF(G7="DNS",0,IF(G7="DQ",0,IF(G7="DNF",1,IF(AND(ISNUMBER(G7),G7&gt;59),1,_xlfn.XLOOKUP(G7,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>44</v>
       </c>
       <c r="J7" s="3" t="str">
         <f>IF(I7="","",IF(I7="DNS",0,IF(I7="DQ",0,IF(I7="DNF",1,IF(AND(ISNUMBER(I7),I7&gt;59),1,_xlfn.XLOOKUP(I7,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -3392,7 +3417,7 @@
       </c>
       <c r="Q7" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="R7" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -3400,7 +3425,7 @@
       </c>
       <c r="S7" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.4">
@@ -3423,9 +3448,12 @@
         <f>IF(E8="","",IF(E8="DNS",0,IF(E8="DQ",0,IF(E8="DNF",1,IF(AND(ISNUMBER(E8),E8&gt;59),1,_xlfn.XLOOKUP(E8,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>43</v>
       </c>
-      <c r="H8" s="3" t="str">
+      <c r="G8" s="3">
+        <v>11</v>
+      </c>
+      <c r="H8" s="3">
         <f>IF(G8="","",IF(G8="DNS",0,IF(G8="DQ",0,IF(G8="DNF",1,IF(AND(ISNUMBER(G8),G8&gt;59),1,_xlfn.XLOOKUP(G8,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>53</v>
       </c>
       <c r="J8" s="3" t="str">
         <f>IF(I8="","",IF(I8="DNS",0,IF(I8="DQ",0,IF(I8="DNF",1,IF(AND(ISNUMBER(I8),I8&gt;59),1,_xlfn.XLOOKUP(I8,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -3445,7 +3473,7 @@
       </c>
       <c r="Q8" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>43</v>
+        <v>96</v>
       </c>
       <c r="R8" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -3453,7 +3481,7 @@
       </c>
       <c r="S8" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>43</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.4">
@@ -3476,9 +3504,12 @@
         <f>IF(E9="","",IF(E9="DNS",0,IF(E9="DQ",0,IF(E9="DNF",1,IF(AND(ISNUMBER(E9),E9&gt;59),1,_xlfn.XLOOKUP(E9,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>22</v>
       </c>
-      <c r="H9" s="3" t="str">
+      <c r="G9" s="3">
+        <v>23</v>
+      </c>
+      <c r="H9" s="3">
         <f>IF(G9="","",IF(G9="DNS",0,IF(G9="DQ",0,IF(G9="DNF",1,IF(AND(ISNUMBER(G9),G9&gt;59),1,_xlfn.XLOOKUP(G9,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>37</v>
       </c>
       <c r="J9" s="3" t="str">
         <f>IF(I9="","",IF(I9="DNS",0,IF(I9="DQ",0,IF(I9="DNF",1,IF(AND(ISNUMBER(I9),I9&gt;59),1,_xlfn.XLOOKUP(I9,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -3498,7 +3529,7 @@
       </c>
       <c r="Q9" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="R9" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -3506,7 +3537,7 @@
       </c>
       <c r="S9" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>22</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.4">
@@ -3529,9 +3560,12 @@
         <f>IF(E10="","",IF(E10="DNS",0,IF(E10="DQ",0,IF(E10="DNF",1,IF(AND(ISNUMBER(E10),E10&gt;59),1,_xlfn.XLOOKUP(E10,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>0</v>
       </c>
-      <c r="H10" s="3" t="str">
+      <c r="G10" s="3">
+        <v>28</v>
+      </c>
+      <c r="H10" s="3">
         <f>IF(G10="","",IF(G10="DNS",0,IF(G10="DQ",0,IF(G10="DNF",1,IF(AND(ISNUMBER(G10),G10&gt;59),1,_xlfn.XLOOKUP(G10,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>32</v>
       </c>
       <c r="J10" s="3" t="str">
         <f>IF(I10="","",IF(I10="DNS",0,IF(I10="DQ",0,IF(I10="DNF",1,IF(AND(ISNUMBER(I10),I10&gt;59),1,_xlfn.XLOOKUP(I10,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -3551,7 +3585,7 @@
       </c>
       <c r="Q10" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="R10" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -3559,7 +3593,7 @@
       </c>
       <c r="S10" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.4">
@@ -3582,9 +3616,12 @@
         <f>IF(E11="","",IF(E11="DNS",0,IF(E11="DQ",0,IF(E11="DNF",1,IF(AND(ISNUMBER(E11),E11&gt;59),1,_xlfn.XLOOKUP(E11,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>36</v>
       </c>
-      <c r="H11" s="3" t="str">
+      <c r="G11" s="3">
+        <v>21</v>
+      </c>
+      <c r="H11" s="3">
         <f>IF(G11="","",IF(G11="DNS",0,IF(G11="DQ",0,IF(G11="DNF",1,IF(AND(ISNUMBER(G11),G11&gt;59),1,_xlfn.XLOOKUP(G11,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>39</v>
       </c>
       <c r="J11" s="3" t="str">
         <f>IF(I11="","",IF(I11="DNS",0,IF(I11="DQ",0,IF(I11="DNF",1,IF(AND(ISNUMBER(I11),I11&gt;59),1,_xlfn.XLOOKUP(I11,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -3604,7 +3641,7 @@
       </c>
       <c r="Q11" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>36</v>
+        <v>75</v>
       </c>
       <c r="R11" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -3612,7 +3649,7 @@
       </c>
       <c r="S11" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>36</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.4">
@@ -3635,9 +3672,12 @@
         <f>IF(E12="","",IF(E12="DNS",0,IF(E12="DQ",0,IF(E12="DNF",1,IF(AND(ISNUMBER(E12),E12&gt;59),1,_xlfn.XLOOKUP(E12,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>29</v>
       </c>
-      <c r="H12" s="3" t="str">
+      <c r="G12" s="3">
+        <v>40</v>
+      </c>
+      <c r="H12" s="3">
         <f>IF(G12="","",IF(G12="DNS",0,IF(G12="DQ",0,IF(G12="DNF",1,IF(AND(ISNUMBER(G12),G12&gt;59),1,_xlfn.XLOOKUP(G12,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>20</v>
       </c>
       <c r="J12" s="3" t="str">
         <f>IF(I12="","",IF(I12="DNS",0,IF(I12="DQ",0,IF(I12="DNF",1,IF(AND(ISNUMBER(I12),I12&gt;59),1,_xlfn.XLOOKUP(I12,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -3657,15 +3697,15 @@
       </c>
       <c r="Q12" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="R12" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="S12" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>29</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.4">
@@ -3688,9 +3728,12 @@
         <f>IF(E13="","",IF(E13="DNS",0,IF(E13="DQ",0,IF(E13="DNF",1,IF(AND(ISNUMBER(E13),E13&gt;59),1,_xlfn.XLOOKUP(E13,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>0</v>
       </c>
-      <c r="H13" s="3" t="str">
+      <c r="G13" s="3">
+        <v>4</v>
+      </c>
+      <c r="H13" s="3">
         <f>IF(G13="","",IF(G13="DNS",0,IF(G13="DQ",0,IF(G13="DNF",1,IF(AND(ISNUMBER(G13),G13&gt;59),1,_xlfn.XLOOKUP(G13,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>85</v>
       </c>
       <c r="J13" s="3" t="str">
         <f>IF(I13="","",IF(I13="DNS",0,IF(I13="DQ",0,IF(I13="DNF",1,IF(AND(ISNUMBER(I13),I13&gt;59),1,_xlfn.XLOOKUP(I13,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -3710,7 +3753,7 @@
       </c>
       <c r="Q13" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="R13" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -3718,7 +3761,7 @@
       </c>
       <c r="S13" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.4">
@@ -3741,9 +3784,12 @@
         <f>IF(E14="","",IF(E14="DNS",0,IF(E14="DQ",0,IF(E14="DNF",1,IF(AND(ISNUMBER(E14),E14&gt;59),1,_xlfn.XLOOKUP(E14,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>0</v>
       </c>
-      <c r="H14" s="3" t="str">
+      <c r="G14" s="3">
+        <v>17</v>
+      </c>
+      <c r="H14" s="3">
         <f>IF(G14="","",IF(G14="DNS",0,IF(G14="DQ",0,IF(G14="DNF",1,IF(AND(ISNUMBER(G14),G14&gt;59),1,_xlfn.XLOOKUP(G14,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>43</v>
       </c>
       <c r="J14" s="3" t="str">
         <f>IF(I14="","",IF(I14="DNS",0,IF(I14="DQ",0,IF(I14="DNF",1,IF(AND(ISNUMBER(I14),I14&gt;59),1,_xlfn.XLOOKUP(I14,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -3763,7 +3809,7 @@
       </c>
       <c r="Q14" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="R14" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -3771,7 +3817,7 @@
       </c>
       <c r="S14" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.4">
@@ -3794,9 +3840,12 @@
         <f>IF(E15="","",IF(E15="DNS",0,IF(E15="DQ",0,IF(E15="DNF",1,IF(AND(ISNUMBER(E15),E15&gt;59),1,_xlfn.XLOOKUP(E15,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>0</v>
       </c>
-      <c r="H15" s="3" t="str">
+      <c r="G15" s="3">
+        <v>41</v>
+      </c>
+      <c r="H15" s="3">
         <f>IF(G15="","",IF(G15="DNS",0,IF(G15="DQ",0,IF(G15="DNF",1,IF(AND(ISNUMBER(G15),G15&gt;59),1,_xlfn.XLOOKUP(G15,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>19</v>
       </c>
       <c r="J15" s="3" t="str">
         <f>IF(I15="","",IF(I15="DNS",0,IF(I15="DQ",0,IF(I15="DNF",1,IF(AND(ISNUMBER(I15),I15&gt;59),1,_xlfn.XLOOKUP(I15,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -3816,7 +3865,7 @@
       </c>
       <c r="Q15" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="R15" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -3824,7 +3873,7 @@
       </c>
       <c r="S15" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.4">
@@ -3847,9 +3896,12 @@
         <f>IF(E16="","",IF(E16="DNS",0,IF(E16="DQ",0,IF(E16="DNF",1,IF(AND(ISNUMBER(E16),E16&gt;59),1,_xlfn.XLOOKUP(E16,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>0</v>
       </c>
-      <c r="H16" s="3" t="str">
+      <c r="G16" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="H16" s="3">
         <f>IF(G16="","",IF(G16="DNS",0,IF(G16="DQ",0,IF(G16="DNF",1,IF(AND(ISNUMBER(G16),G16&gt;59),1,_xlfn.XLOOKUP(G16,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J16" s="3" t="str">
         <f>IF(I16="","",IF(I16="DNS",0,IF(I16="DQ",0,IF(I16="DNF",1,IF(AND(ISNUMBER(I16),I16&gt;59),1,_xlfn.XLOOKUP(I16,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -3900,9 +3952,12 @@
         <f>IF(E17="","",IF(E17="DNS",0,IF(E17="DQ",0,IF(E17="DNF",1,IF(AND(ISNUMBER(E17),E17&gt;59),1,_xlfn.XLOOKUP(E17,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>70</v>
       </c>
-      <c r="H17" s="3" t="str">
+      <c r="G17" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="H17" s="3">
         <f>IF(G17="","",IF(G17="DNS",0,IF(G17="DQ",0,IF(G17="DNF",1,IF(AND(ISNUMBER(G17),G17&gt;59),1,_xlfn.XLOOKUP(G17,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J17" s="3" t="str">
         <f>IF(I17="","",IF(I17="DNS",0,IF(I17="DQ",0,IF(I17="DNF",1,IF(AND(ISNUMBER(I17),I17&gt;59),1,_xlfn.XLOOKUP(I17,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -3926,7 +3981,7 @@
       </c>
       <c r="R17" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="S17" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
@@ -3953,9 +4008,12 @@
         <f>IF(E18="","",IF(E18="DNS",0,IF(E18="DQ",0,IF(E18="DNF",1,IF(AND(ISNUMBER(E18),E18&gt;59),1,_xlfn.XLOOKUP(E18,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>0</v>
       </c>
-      <c r="H18" s="3" t="str">
+      <c r="G18" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="H18" s="3">
         <f>IF(G18="","",IF(G18="DNS",0,IF(G18="DQ",0,IF(G18="DNF",1,IF(AND(ISNUMBER(G18),G18&gt;59),1,_xlfn.XLOOKUP(G18,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J18" s="3" t="str">
         <f>IF(I18="","",IF(I18="DNS",0,IF(I18="DQ",0,IF(I18="DNF",1,IF(AND(ISNUMBER(I18),I18&gt;59),1,_xlfn.XLOOKUP(I18,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -4006,9 +4064,12 @@
         <f>IF(E19="","",IF(E19="DNS",0,IF(E19="DQ",0,IF(E19="DNF",1,IF(AND(ISNUMBER(E19),E19&gt;59),1,_xlfn.XLOOKUP(E19,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>0</v>
       </c>
-      <c r="H19" s="3" t="str">
+      <c r="G19" s="3">
+        <v>2</v>
+      </c>
+      <c r="H19" s="3">
         <f>IF(G19="","",IF(G19="DNS",0,IF(G19="DQ",0,IF(G19="DNF",1,IF(AND(ISNUMBER(G19),G19&gt;59),1,_xlfn.XLOOKUP(G19,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>95</v>
       </c>
       <c r="J19" s="3" t="str">
         <f>IF(I19="","",IF(I19="DNS",0,IF(I19="DQ",0,IF(I19="DNF",1,IF(AND(ISNUMBER(I19),I19&gt;59),1,_xlfn.XLOOKUP(I19,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -4028,7 +4089,7 @@
       </c>
       <c r="Q19" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="R19" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -4036,7 +4097,7 @@
       </c>
       <c r="S19" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>95</v>
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.4">
@@ -4059,9 +4120,12 @@
         <f>IF(E20="","",IF(E20="DNS",0,IF(E20="DQ",0,IF(E20="DNF",1,IF(AND(ISNUMBER(E20),E20&gt;59),1,_xlfn.XLOOKUP(E20,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>90</v>
       </c>
-      <c r="H20" s="3" t="str">
+      <c r="G20" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="H20" s="3">
         <f>IF(G20="","",IF(G20="DNS",0,IF(G20="DQ",0,IF(G20="DNF",1,IF(AND(ISNUMBER(G20),G20&gt;59),1,_xlfn.XLOOKUP(G20,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J20" s="3" t="str">
         <f>IF(I20="","",IF(I20="DNS",0,IF(I20="DQ",0,IF(I20="DNF",1,IF(AND(ISNUMBER(I20),I20&gt;59),1,_xlfn.XLOOKUP(I20,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -4085,7 +4149,7 @@
       </c>
       <c r="R20" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="S20" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
@@ -4112,9 +4176,12 @@
         <f>IF(E21="","",IF(E21="DNS",0,IF(E21="DQ",0,IF(E21="DNF",1,IF(AND(ISNUMBER(E21),E21&gt;59),1,_xlfn.XLOOKUP(E21,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>19</v>
       </c>
-      <c r="H21" s="3" t="str">
+      <c r="G21" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="H21" s="3">
         <f>IF(G21="","",IF(G21="DNS",0,IF(G21="DQ",0,IF(G21="DNF",1,IF(AND(ISNUMBER(G21),G21&gt;59),1,_xlfn.XLOOKUP(G21,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J21" s="3" t="str">
         <f>IF(I21="","",IF(I21="DNS",0,IF(I21="DQ",0,IF(I21="DNF",1,IF(AND(ISNUMBER(I21),I21&gt;59),1,_xlfn.XLOOKUP(I21,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -4138,7 +4205,7 @@
       </c>
       <c r="R21" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="S21" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
@@ -4165,9 +4232,12 @@
         <f>IF(E22="","",IF(E22="DNS",0,IF(E22="DQ",0,IF(E22="DNF",1,IF(AND(ISNUMBER(E22),E22&gt;59),1,_xlfn.XLOOKUP(E22,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>44</v>
       </c>
-      <c r="H22" s="3" t="str">
+      <c r="G22" s="3">
+        <v>12</v>
+      </c>
+      <c r="H22" s="3">
         <f>IF(G22="","",IF(G22="DNS",0,IF(G22="DQ",0,IF(G22="DNF",1,IF(AND(ISNUMBER(G22),G22&gt;59),1,_xlfn.XLOOKUP(G22,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>51</v>
       </c>
       <c r="J22" s="3" t="str">
         <f>IF(I22="","",IF(I22="DNS",0,IF(I22="DQ",0,IF(I22="DNF",1,IF(AND(ISNUMBER(I22),I22&gt;59),1,_xlfn.XLOOKUP(I22,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -4187,7 +4257,7 @@
       </c>
       <c r="Q22" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>44</v>
+        <v>95</v>
       </c>
       <c r="R22" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -4195,7 +4265,7 @@
       </c>
       <c r="S22" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>44</v>
+        <v>95</v>
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.4">
@@ -4218,9 +4288,12 @@
         <f>IF(E23="","",IF(E23="DNS",0,IF(E23="DQ",0,IF(E23="DNF",1,IF(AND(ISNUMBER(E23),E23&gt;59),1,_xlfn.XLOOKUP(E23,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>27</v>
       </c>
-      <c r="H23" s="3" t="str">
+      <c r="G23" s="3">
+        <v>6</v>
+      </c>
+      <c r="H23" s="3">
         <f>IF(G23="","",IF(G23="DNS",0,IF(G23="DQ",0,IF(G23="DNF",1,IF(AND(ISNUMBER(G23),G23&gt;59),1,_xlfn.XLOOKUP(G23,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>75</v>
       </c>
       <c r="J23" s="3" t="str">
         <f>IF(I23="","",IF(I23="DNS",0,IF(I23="DQ",0,IF(I23="DNF",1,IF(AND(ISNUMBER(I23),I23&gt;59),1,_xlfn.XLOOKUP(I23,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -4240,7 +4313,7 @@
       </c>
       <c r="Q23" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>27</v>
+        <v>102</v>
       </c>
       <c r="R23" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -4248,7 +4321,7 @@
       </c>
       <c r="S23" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>27</v>
+        <v>102</v>
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.4">
@@ -4271,9 +4344,12 @@
         <f>IF(E24="","",IF(E24="DNS",0,IF(E24="DQ",0,IF(E24="DNF",1,IF(AND(ISNUMBER(E24),E24&gt;59),1,_xlfn.XLOOKUP(E24,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>51</v>
       </c>
-      <c r="H24" s="3" t="str">
+      <c r="G24" s="3">
+        <v>39</v>
+      </c>
+      <c r="H24" s="3">
         <f>IF(G24="","",IF(G24="DNS",0,IF(G24="DQ",0,IF(G24="DNF",1,IF(AND(ISNUMBER(G24),G24&gt;59),1,_xlfn.XLOOKUP(G24,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>21</v>
       </c>
       <c r="J24" s="3" t="str">
         <f>IF(I24="","",IF(I24="DNS",0,IF(I24="DQ",0,IF(I24="DNF",1,IF(AND(ISNUMBER(I24),I24&gt;59),1,_xlfn.XLOOKUP(I24,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -4293,15 +4369,15 @@
       </c>
       <c r="Q24" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>51</v>
+        <v>72</v>
       </c>
       <c r="R24" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="S24" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>51</v>
+        <v>72</v>
       </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.4">
@@ -4324,9 +4400,12 @@
         <f>IF(E25="","",IF(E25="DNS",0,IF(E25="DQ",0,IF(E25="DNF",1,IF(AND(ISNUMBER(E25),E25&gt;59),1,_xlfn.XLOOKUP(E25,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>1</v>
       </c>
-      <c r="H25" s="3" t="str">
+      <c r="G25" s="3">
+        <v>9</v>
+      </c>
+      <c r="H25" s="3">
         <f>IF(G25="","",IF(G25="DNS",0,IF(G25="DQ",0,IF(G25="DNF",1,IF(AND(ISNUMBER(G25),G25&gt;59),1,_xlfn.XLOOKUP(G25,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>60</v>
       </c>
       <c r="J25" s="3" t="str">
         <f>IF(I25="","",IF(I25="DNS",0,IF(I25="DQ",0,IF(I25="DNF",1,IF(AND(ISNUMBER(I25),I25&gt;59),1,_xlfn.XLOOKUP(I25,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -4346,7 +4425,7 @@
       </c>
       <c r="Q25" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>1</v>
+        <v>61</v>
       </c>
       <c r="R25" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -4354,7 +4433,7 @@
       </c>
       <c r="S25" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>1</v>
+        <v>61</v>
       </c>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.4">
@@ -4377,9 +4456,12 @@
         <f>IF(E26="","",IF(E26="DNS",0,IF(E26="DQ",0,IF(E26="DNF",1,IF(AND(ISNUMBER(E26),E26&gt;59),1,_xlfn.XLOOKUP(E26,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>60</v>
       </c>
-      <c r="H26" s="3" t="str">
+      <c r="G26" s="3">
+        <v>42</v>
+      </c>
+      <c r="H26" s="3">
         <f>IF(G26="","",IF(G26="DNS",0,IF(G26="DQ",0,IF(G26="DNF",1,IF(AND(ISNUMBER(G26),G26&gt;59),1,_xlfn.XLOOKUP(G26,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>18</v>
       </c>
       <c r="J26" s="3" t="str">
         <f>IF(I26="","",IF(I26="DNS",0,IF(I26="DQ",0,IF(I26="DNF",1,IF(AND(ISNUMBER(I26),I26&gt;59),1,_xlfn.XLOOKUP(I26,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -4399,15 +4481,15 @@
       </c>
       <c r="Q26" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="R26" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="S26" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>60</v>
+        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.4">
@@ -4430,9 +4512,12 @@
         <f>IF(E27="","",IF(E27="DNS",0,IF(E27="DQ",0,IF(E27="DNF",1,IF(AND(ISNUMBER(E27),E27&gt;59),1,_xlfn.XLOOKUP(E27,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>26</v>
       </c>
-      <c r="H27" s="3" t="str">
+      <c r="G27" s="3">
+        <v>36</v>
+      </c>
+      <c r="H27" s="3">
         <f>IF(G27="","",IF(G27="DNS",0,IF(G27="DQ",0,IF(G27="DNF",1,IF(AND(ISNUMBER(G27),G27&gt;59),1,_xlfn.XLOOKUP(G27,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>24</v>
       </c>
       <c r="J27" s="3" t="str">
         <f>IF(I27="","",IF(I27="DNS",0,IF(I27="DQ",0,IF(I27="DNF",1,IF(AND(ISNUMBER(I27),I27&gt;59),1,_xlfn.XLOOKUP(I27,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -4452,15 +4537,15 @@
       </c>
       <c r="Q27" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="R27" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="S27" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>26</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.4">
@@ -4483,9 +4568,12 @@
         <f>IF(E28="","",IF(E28="DNS",0,IF(E28="DQ",0,IF(E28="DNF",1,IF(AND(ISNUMBER(E28),E28&gt;59),1,_xlfn.XLOOKUP(E28,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>0</v>
       </c>
-      <c r="H28" s="3" t="str">
+      <c r="G28" s="3">
+        <v>19</v>
+      </c>
+      <c r="H28" s="3">
         <f>IF(G28="","",IF(G28="DNS",0,IF(G28="DQ",0,IF(G28="DNF",1,IF(AND(ISNUMBER(G28),G28&gt;59),1,_xlfn.XLOOKUP(G28,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>41</v>
       </c>
       <c r="J28" s="3" t="str">
         <f>IF(I28="","",IF(I28="DNS",0,IF(I28="DQ",0,IF(I28="DNF",1,IF(AND(ISNUMBER(I28),I28&gt;59),1,_xlfn.XLOOKUP(I28,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -4505,7 +4593,7 @@
       </c>
       <c r="Q28" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="R28" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -4513,7 +4601,7 @@
       </c>
       <c r="S28" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>41</v>
       </c>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.4">
@@ -4536,9 +4624,12 @@
         <f>IF(E29="","",IF(E29="DNS",0,IF(E29="DQ",0,IF(E29="DNF",1,IF(AND(ISNUMBER(E29),E29&gt;59),1,_xlfn.XLOOKUP(E29,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>0</v>
       </c>
-      <c r="H29" s="3" t="str">
+      <c r="G29" s="3">
+        <v>14</v>
+      </c>
+      <c r="H29" s="3">
         <f>IF(G29="","",IF(G29="DNS",0,IF(G29="DQ",0,IF(G29="DNF",1,IF(AND(ISNUMBER(G29),G29&gt;59),1,_xlfn.XLOOKUP(G29,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>47</v>
       </c>
       <c r="J29" s="3" t="str">
         <f>IF(I29="","",IF(I29="DNS",0,IF(I29="DQ",0,IF(I29="DNF",1,IF(AND(ISNUMBER(I29),I29&gt;59),1,_xlfn.XLOOKUP(I29,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -4558,7 +4649,7 @@
       </c>
       <c r="Q29" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="R29" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -4566,7 +4657,7 @@
       </c>
       <c r="S29" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>47</v>
       </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.4">
@@ -4589,9 +4680,12 @@
         <f>IF(E30="","",IF(E30="DNS",0,IF(E30="DQ",0,IF(E30="DNF",1,IF(AND(ISNUMBER(E30),E30&gt;59),1,_xlfn.XLOOKUP(E30,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>100</v>
       </c>
-      <c r="H30" s="3" t="str">
+      <c r="G30" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="H30" s="3">
         <f>IF(G30="","",IF(G30="DNS",0,IF(G30="DQ",0,IF(G30="DNF",1,IF(AND(ISNUMBER(G30),G30&gt;59),1,_xlfn.XLOOKUP(G30,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J30" s="3" t="str">
         <f>IF(I30="","",IF(I30="DNS",0,IF(I30="DQ",0,IF(I30="DNF",1,IF(AND(ISNUMBER(I30),I30&gt;59),1,_xlfn.XLOOKUP(I30,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -4615,7 +4709,7 @@
       </c>
       <c r="R30" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="S30" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
@@ -4642,9 +4736,12 @@
         <f>IF(E31="","",IF(E31="DNS",0,IF(E31="DQ",0,IF(E31="DNF",1,IF(AND(ISNUMBER(E31),E31&gt;59),1,_xlfn.XLOOKUP(E31,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>18</v>
       </c>
-      <c r="H31" s="3" t="str">
+      <c r="G31" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="H31" s="3">
         <f>IF(G31="","",IF(G31="DNS",0,IF(G31="DQ",0,IF(G31="DNF",1,IF(AND(ISNUMBER(G31),G31&gt;59),1,_xlfn.XLOOKUP(G31,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J31" s="3" t="str">
         <f>IF(I31="","",IF(I31="DNS",0,IF(I31="DQ",0,IF(I31="DNF",1,IF(AND(ISNUMBER(I31),I31&gt;59),1,_xlfn.XLOOKUP(I31,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -4668,7 +4765,7 @@
       </c>
       <c r="R31" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="S31" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
@@ -4695,9 +4792,12 @@
         <f>IF(E32="","",IF(E32="DNS",0,IF(E32="DQ",0,IF(E32="DNF",1,IF(AND(ISNUMBER(E32),E32&gt;59),1,_xlfn.XLOOKUP(E32,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>28</v>
       </c>
-      <c r="H32" s="3" t="str">
+      <c r="G32" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="H32" s="3">
         <f>IF(G32="","",IF(G32="DNS",0,IF(G32="DQ",0,IF(G32="DNF",1,IF(AND(ISNUMBER(G32),G32&gt;59),1,_xlfn.XLOOKUP(G32,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J32" s="3" t="str">
         <f>IF(I32="","",IF(I32="DNS",0,IF(I32="DQ",0,IF(I32="DNF",1,IF(AND(ISNUMBER(I32),I32&gt;59),1,_xlfn.XLOOKUP(I32,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -4721,7 +4821,7 @@
       </c>
       <c r="R32" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="S32" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
@@ -4748,9 +4848,12 @@
         <f>IF(E33="","",IF(E33="DNS",0,IF(E33="DQ",0,IF(E33="DNF",1,IF(AND(ISNUMBER(E33),E33&gt;59),1,_xlfn.XLOOKUP(E33,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>25</v>
       </c>
-      <c r="H33" s="3" t="str">
+      <c r="G33" s="3">
+        <v>8</v>
+      </c>
+      <c r="H33" s="3">
         <f>IF(G33="","",IF(G33="DNS",0,IF(G33="DQ",0,IF(G33="DNF",1,IF(AND(ISNUMBER(G33),G33&gt;59),1,_xlfn.XLOOKUP(G33,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>65</v>
       </c>
       <c r="J33" s="3" t="str">
         <f>IF(I33="","",IF(I33="DNS",0,IF(I33="DQ",0,IF(I33="DNF",1,IF(AND(ISNUMBER(I33),I33&gt;59),1,_xlfn.XLOOKUP(I33,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -4770,7 +4873,7 @@
       </c>
       <c r="Q33" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>25</v>
+        <v>90</v>
       </c>
       <c r="R33" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -4778,7 +4881,7 @@
       </c>
       <c r="S33" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>25</v>
+        <v>90</v>
       </c>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.4">
@@ -4801,9 +4904,12 @@
         <f>IF(E34="","",IF(E34="DNS",0,IF(E34="DQ",0,IF(E34="DNF",1,IF(AND(ISNUMBER(E34),E34&gt;59),1,_xlfn.XLOOKUP(E34,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>47</v>
       </c>
-      <c r="H34" s="3" t="str">
+      <c r="G34" s="3">
+        <v>38</v>
+      </c>
+      <c r="H34" s="3">
         <f>IF(G34="","",IF(G34="DNS",0,IF(G34="DQ",0,IF(G34="DNF",1,IF(AND(ISNUMBER(G34),G34&gt;59),1,_xlfn.XLOOKUP(G34,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>22</v>
       </c>
       <c r="J34" s="3" t="str">
         <f>IF(I34="","",IF(I34="DNS",0,IF(I34="DQ",0,IF(I34="DNF",1,IF(AND(ISNUMBER(I34),I34&gt;59),1,_xlfn.XLOOKUP(I34,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -4823,15 +4929,15 @@
       </c>
       <c r="Q34" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>47</v>
+        <v>69</v>
       </c>
       <c r="R34" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="S34" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>47</v>
+        <v>69</v>
       </c>
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.4">
@@ -4854,9 +4960,12 @@
         <f>IF(E35="","",IF(E35="DNS",0,IF(E35="DQ",0,IF(E35="DNF",1,IF(AND(ISNUMBER(E35),E35&gt;59),1,_xlfn.XLOOKUP(E35,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>38</v>
       </c>
-      <c r="H35" s="3" t="str">
+      <c r="G35" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="H35" s="3">
         <f>IF(G35="","",IF(G35="DNS",0,IF(G35="DQ",0,IF(G35="DNF",1,IF(AND(ISNUMBER(G35),G35&gt;59),1,_xlfn.XLOOKUP(G35,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J35" s="3" t="str">
         <f>IF(I35="","",IF(I35="DNS",0,IF(I35="DQ",0,IF(I35="DNF",1,IF(AND(ISNUMBER(I35),I35&gt;59),1,_xlfn.XLOOKUP(I35,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -4880,7 +4989,7 @@
       </c>
       <c r="R35" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="S35" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
@@ -4907,9 +5016,12 @@
         <f>IF(E36="","",IF(E36="DNS",0,IF(E36="DQ",0,IF(E36="DNF",1,IF(AND(ISNUMBER(E36),E36&gt;59),1,_xlfn.XLOOKUP(E36,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>53</v>
       </c>
-      <c r="H36" s="3" t="str">
+      <c r="G36" s="3">
+        <v>29</v>
+      </c>
+      <c r="H36" s="3">
         <f>IF(G36="","",IF(G36="DNS",0,IF(G36="DQ",0,IF(G36="DNF",1,IF(AND(ISNUMBER(G36),G36&gt;59),1,_xlfn.XLOOKUP(G36,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>31</v>
       </c>
       <c r="J36" s="3" t="str">
         <f>IF(I36="","",IF(I36="DNS",0,IF(I36="DQ",0,IF(I36="DNF",1,IF(AND(ISNUMBER(I36),I36&gt;59),1,_xlfn.XLOOKUP(I36,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -4929,15 +5041,15 @@
       </c>
       <c r="Q36" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="R36" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="S36" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>53</v>
+        <v>84</v>
       </c>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.4">
@@ -4960,9 +5072,12 @@
         <f>IF(E37="","",IF(E37="DNS",0,IF(E37="DQ",0,IF(E37="DNF",1,IF(AND(ISNUMBER(E37),E37&gt;59),1,_xlfn.XLOOKUP(E37,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>30</v>
       </c>
-      <c r="H37" s="3" t="str">
+      <c r="G37" s="3">
+        <v>13</v>
+      </c>
+      <c r="H37" s="3">
         <f>IF(G37="","",IF(G37="DNS",0,IF(G37="DQ",0,IF(G37="DNF",1,IF(AND(ISNUMBER(G37),G37&gt;59),1,_xlfn.XLOOKUP(G37,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>49</v>
       </c>
       <c r="J37" s="3" t="str">
         <f>IF(I37="","",IF(I37="DNS",0,IF(I37="DQ",0,IF(I37="DNF",1,IF(AND(ISNUMBER(I37),I37&gt;59),1,_xlfn.XLOOKUP(I37,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -4982,7 +5097,7 @@
       </c>
       <c r="Q37" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="R37" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -4990,7 +5105,7 @@
       </c>
       <c r="S37" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>30</v>
+        <v>79</v>
       </c>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.4">
@@ -5013,9 +5128,12 @@
         <f>IF(E38="","",IF(E38="DNS",0,IF(E38="DQ",0,IF(E38="DNF",1,IF(AND(ISNUMBER(E38),E38&gt;59),1,_xlfn.XLOOKUP(E38,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>0</v>
       </c>
-      <c r="H38" s="3" t="str">
+      <c r="G38" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="H38" s="3">
         <f>IF(G38="","",IF(G38="DNS",0,IF(G38="DQ",0,IF(G38="DNF",1,IF(AND(ISNUMBER(G38),G38&gt;59),1,_xlfn.XLOOKUP(G38,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J38" s="3" t="str">
         <f>IF(I38="","",IF(I38="DNS",0,IF(I38="DQ",0,IF(I38="DNF",1,IF(AND(ISNUMBER(I38),I38&gt;59),1,_xlfn.XLOOKUP(I38,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -5066,9 +5184,12 @@
         <f>IF(E39="","",IF(E39="DNS",0,IF(E39="DQ",0,IF(E39="DNF",1,IF(AND(ISNUMBER(E39),E39&gt;59),1,_xlfn.XLOOKUP(E39,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>65</v>
       </c>
-      <c r="H39" s="3" t="str">
+      <c r="G39" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="H39" s="3">
         <f>IF(G39="","",IF(G39="DNS",0,IF(G39="DQ",0,IF(G39="DNF",1,IF(AND(ISNUMBER(G39),G39&gt;59),1,_xlfn.XLOOKUP(G39,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J39" s="3" t="str">
         <f>IF(I39="","",IF(I39="DNS",0,IF(I39="DQ",0,IF(I39="DNF",1,IF(AND(ISNUMBER(I39),I39&gt;59),1,_xlfn.XLOOKUP(I39,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -5092,7 +5213,7 @@
       </c>
       <c r="R39" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="S39" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
@@ -5119,9 +5240,12 @@
         <f>IF(E40="","",IF(E40="DNS",0,IF(E40="DQ",0,IF(E40="DNF",1,IF(AND(ISNUMBER(E40),E40&gt;59),1,_xlfn.XLOOKUP(E40,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>37</v>
       </c>
-      <c r="H40" s="3" t="str">
+      <c r="G40" s="3">
+        <v>31</v>
+      </c>
+      <c r="H40" s="3">
         <f>IF(G40="","",IF(G40="DNS",0,IF(G40="DQ",0,IF(G40="DNF",1,IF(AND(ISNUMBER(G40),G40&gt;59),1,_xlfn.XLOOKUP(G40,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>29</v>
       </c>
       <c r="J40" s="3" t="str">
         <f>IF(I40="","",IF(I40="DNS",0,IF(I40="DQ",0,IF(I40="DNF",1,IF(AND(ISNUMBER(I40),I40&gt;59),1,_xlfn.XLOOKUP(I40,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -5141,15 +5265,15 @@
       </c>
       <c r="Q40" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>37</v>
+        <v>66</v>
       </c>
       <c r="R40" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="S40" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>37</v>
+        <v>66</v>
       </c>
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.4">
@@ -5172,9 +5296,12 @@
         <f>IF(E41="","",IF(E41="DNS",0,IF(E41="DQ",0,IF(E41="DNF",1,IF(AND(ISNUMBER(E41),E41&gt;59),1,_xlfn.XLOOKUP(E41,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>55</v>
       </c>
-      <c r="H41" s="3" t="str">
+      <c r="G41" s="3">
+        <v>30</v>
+      </c>
+      <c r="H41" s="3">
         <f>IF(G41="","",IF(G41="DNS",0,IF(G41="DQ",0,IF(G41="DNF",1,IF(AND(ISNUMBER(G41),G41&gt;59),1,_xlfn.XLOOKUP(G41,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>30</v>
       </c>
       <c r="J41" s="3" t="str">
         <f>IF(I41="","",IF(I41="DNS",0,IF(I41="DQ",0,IF(I41="DNF",1,IF(AND(ISNUMBER(I41),I41&gt;59),1,_xlfn.XLOOKUP(I41,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -5194,15 +5321,15 @@
       </c>
       <c r="Q41" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>55</v>
+        <v>85</v>
       </c>
       <c r="R41" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="S41" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>55</v>
+        <v>85</v>
       </c>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.4">
@@ -5225,9 +5352,12 @@
         <f>IF(E42="","",IF(E42="DNS",0,IF(E42="DQ",0,IF(E42="DNF",1,IF(AND(ISNUMBER(E42),E42&gt;59),1,_xlfn.XLOOKUP(E42,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>32</v>
       </c>
-      <c r="H42" s="3" t="str">
+      <c r="G42" s="3">
+        <v>27</v>
+      </c>
+      <c r="H42" s="3">
         <f>IF(G42="","",IF(G42="DNS",0,IF(G42="DQ",0,IF(G42="DNF",1,IF(AND(ISNUMBER(G42),G42&gt;59),1,_xlfn.XLOOKUP(G42,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>33</v>
       </c>
       <c r="J42" s="3" t="str">
         <f>IF(I42="","",IF(I42="DNS",0,IF(I42="DQ",0,IF(I42="DNF",1,IF(AND(ISNUMBER(I42),I42&gt;59),1,_xlfn.XLOOKUP(I42,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -5247,7 +5377,7 @@
       </c>
       <c r="Q42" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>32</v>
+        <v>65</v>
       </c>
       <c r="R42" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -5255,7 +5385,7 @@
       </c>
       <c r="S42" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>32</v>
+        <v>65</v>
       </c>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.4">
@@ -5278,9 +5408,12 @@
         <f>IF(E43="","",IF(E43="DNS",0,IF(E43="DQ",0,IF(E43="DNF",1,IF(AND(ISNUMBER(E43),E43&gt;59),1,_xlfn.XLOOKUP(E43,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>80</v>
       </c>
-      <c r="H43" s="3" t="str">
+      <c r="G43" s="3">
+        <v>35</v>
+      </c>
+      <c r="H43" s="3">
         <f>IF(G43="","",IF(G43="DNS",0,IF(G43="DQ",0,IF(G43="DNF",1,IF(AND(ISNUMBER(G43),G43&gt;59),1,_xlfn.XLOOKUP(G43,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>25</v>
       </c>
       <c r="J43" s="3" t="str">
         <f>IF(I43="","",IF(I43="DNS",0,IF(I43="DQ",0,IF(I43="DNF",1,IF(AND(ISNUMBER(I43),I43&gt;59),1,_xlfn.XLOOKUP(I43,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -5300,15 +5433,15 @@
       </c>
       <c r="Q43" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>80</v>
+        <v>105</v>
       </c>
       <c r="R43" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>80</v>
+        <v>25</v>
       </c>
       <c r="S43" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>80</v>
+        <v>105</v>
       </c>
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.4">
@@ -5331,9 +5464,12 @@
         <f>IF(E44="","",IF(E44="DNS",0,IF(E44="DQ",0,IF(E44="DNF",1,IF(AND(ISNUMBER(E44),E44&gt;59),1,_xlfn.XLOOKUP(E44,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>31</v>
       </c>
-      <c r="H44" s="3" t="str">
+      <c r="G44" s="3">
+        <v>10</v>
+      </c>
+      <c r="H44" s="3">
         <f>IF(G44="","",IF(G44="DNS",0,IF(G44="DQ",0,IF(G44="DNF",1,IF(AND(ISNUMBER(G44),G44&gt;59),1,_xlfn.XLOOKUP(G44,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>55</v>
       </c>
       <c r="J44" s="3" t="str">
         <f>IF(I44="","",IF(I44="DNS",0,IF(I44="DQ",0,IF(I44="DNF",1,IF(AND(ISNUMBER(I44),I44&gt;59),1,_xlfn.XLOOKUP(I44,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -5353,7 +5489,7 @@
       </c>
       <c r="Q44" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>31</v>
+        <v>86</v>
       </c>
       <c r="R44" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -5361,7 +5497,7 @@
       </c>
       <c r="S44" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>31</v>
+        <v>86</v>
       </c>
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.4">
@@ -5384,9 +5520,12 @@
         <f>IF(E45="","",IF(E45="DNS",0,IF(E45="DQ",0,IF(E45="DNF",1,IF(AND(ISNUMBER(E45),E45&gt;59),1,_xlfn.XLOOKUP(E45,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>75</v>
       </c>
-      <c r="H45" s="3" t="str">
+      <c r="G45" s="3">
+        <v>46</v>
+      </c>
+      <c r="H45" s="3">
         <f>IF(G45="","",IF(G45="DNS",0,IF(G45="DQ",0,IF(G45="DNF",1,IF(AND(ISNUMBER(G45),G45&gt;59),1,_xlfn.XLOOKUP(G45,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>14</v>
       </c>
       <c r="J45" s="3" t="str">
         <f>IF(I45="","",IF(I45="DNS",0,IF(I45="DQ",0,IF(I45="DNF",1,IF(AND(ISNUMBER(I45),I45&gt;59),1,_xlfn.XLOOKUP(I45,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -5406,15 +5545,15 @@
       </c>
       <c r="Q45" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="R45" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>75</v>
+        <v>14</v>
       </c>
       <c r="S45" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>75</v>
+        <v>89</v>
       </c>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.4">
@@ -5437,9 +5576,12 @@
         <f>IF(E46="","",IF(E46="DNS",0,IF(E46="DQ",0,IF(E46="DNF",1,IF(AND(ISNUMBER(E46),E46&gt;59),1,_xlfn.XLOOKUP(E46,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>20</v>
       </c>
-      <c r="H46" s="3" t="str">
+      <c r="G46" s="3">
+        <v>3</v>
+      </c>
+      <c r="H46" s="3">
         <f>IF(G46="","",IF(G46="DNS",0,IF(G46="DQ",0,IF(G46="DNF",1,IF(AND(ISNUMBER(G46),G46&gt;59),1,_xlfn.XLOOKUP(G46,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>90</v>
       </c>
       <c r="J46" s="3" t="str">
         <f>IF(I46="","",IF(I46="DNS",0,IF(I46="DQ",0,IF(I46="DNF",1,IF(AND(ISNUMBER(I46),I46&gt;59),1,_xlfn.XLOOKUP(I46,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -5459,7 +5601,7 @@
       </c>
       <c r="Q46" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>20</v>
+        <v>110</v>
       </c>
       <c r="R46" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -5467,7 +5609,7 @@
       </c>
       <c r="S46" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>20</v>
+        <v>110</v>
       </c>
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.4">
@@ -5490,9 +5632,12 @@
         <f>IF(E47="","",IF(E47="DNS",0,IF(E47="DQ",0,IF(E47="DNF",1,IF(AND(ISNUMBER(E47),E47&gt;59),1,_xlfn.XLOOKUP(E47,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>33</v>
       </c>
-      <c r="H47" s="3" t="str">
+      <c r="G47" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="H47" s="3">
         <f>IF(G47="","",IF(G47="DNS",0,IF(G47="DQ",0,IF(G47="DNF",1,IF(AND(ISNUMBER(G47),G47&gt;59),1,_xlfn.XLOOKUP(G47,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J47" s="3" t="str">
         <f>IF(I47="","",IF(I47="DNS",0,IF(I47="DQ",0,IF(I47="DNF",1,IF(AND(ISNUMBER(I47),I47&gt;59),1,_xlfn.XLOOKUP(I47,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -5516,7 +5661,7 @@
       </c>
       <c r="R47" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="S47" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
@@ -5543,9 +5688,12 @@
         <f>IF(E48="","",IF(E48="DNS",0,IF(E48="DQ",0,IF(E48="DNF",1,IF(AND(ISNUMBER(E48),E48&gt;59),1,_xlfn.XLOOKUP(E48,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>40</v>
       </c>
-      <c r="H48" s="3" t="str">
+      <c r="G48" s="3">
+        <v>7</v>
+      </c>
+      <c r="H48" s="3">
         <f>IF(G48="","",IF(G48="DNS",0,IF(G48="DQ",0,IF(G48="DNF",1,IF(AND(ISNUMBER(G48),G48&gt;59),1,_xlfn.XLOOKUP(G48,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>70</v>
       </c>
       <c r="J48" s="3" t="str">
         <f>IF(I48="","",IF(I48="DNS",0,IF(I48="DQ",0,IF(I48="DNF",1,IF(AND(ISNUMBER(I48),I48&gt;59),1,_xlfn.XLOOKUP(I48,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -5565,7 +5713,7 @@
       </c>
       <c r="Q48" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>40</v>
+        <v>110</v>
       </c>
       <c r="R48" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -5573,7 +5721,7 @@
       </c>
       <c r="S48" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>40</v>
+        <v>110</v>
       </c>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.4">
@@ -5596,9 +5744,12 @@
         <f>IF(E49="","",IF(E49="DNS",0,IF(E49="DQ",0,IF(E49="DNF",1,IF(AND(ISNUMBER(E49),E49&gt;59),1,_xlfn.XLOOKUP(E49,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>23</v>
       </c>
-      <c r="H49" s="3" t="str">
+      <c r="G49" s="3">
+        <v>43</v>
+      </c>
+      <c r="H49" s="3">
         <f>IF(G49="","",IF(G49="DNS",0,IF(G49="DQ",0,IF(G49="DNF",1,IF(AND(ISNUMBER(G49),G49&gt;59),1,_xlfn.XLOOKUP(G49,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>17</v>
       </c>
       <c r="J49" s="3" t="str">
         <f>IF(I49="","",IF(I49="DNS",0,IF(I49="DQ",0,IF(I49="DNF",1,IF(AND(ISNUMBER(I49),I49&gt;59),1,_xlfn.XLOOKUP(I49,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -5618,15 +5769,15 @@
       </c>
       <c r="Q49" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="R49" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="S49" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>23</v>
+        <v>40</v>
       </c>
     </row>
     <row r="50" spans="1:19" x14ac:dyDescent="0.4">
@@ -5649,9 +5800,12 @@
         <f>IF(E50="","",IF(E50="DNS",0,IF(E50="DQ",0,IF(E50="DNF",1,IF(AND(ISNUMBER(E50),E50&gt;59),1,_xlfn.XLOOKUP(E50,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>41</v>
       </c>
-      <c r="H50" s="3" t="str">
+      <c r="G50" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="H50" s="3">
         <f>IF(G50="","",IF(G50="DNS",0,IF(G50="DQ",0,IF(G50="DNF",1,IF(AND(ISNUMBER(G50),G50&gt;59),1,_xlfn.XLOOKUP(G50,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J50" s="3" t="str">
         <f>IF(I50="","",IF(I50="DNS",0,IF(I50="DQ",0,IF(I50="DNF",1,IF(AND(ISNUMBER(I50),I50&gt;59),1,_xlfn.XLOOKUP(I50,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -5675,7 +5829,7 @@
       </c>
       <c r="R50" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="S50" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
@@ -5702,9 +5856,12 @@
         <f>IF(E51="","",IF(E51="DNS",0,IF(E51="DQ",0,IF(E51="DNF",1,IF(AND(ISNUMBER(E51),E51&gt;59),1,_xlfn.XLOOKUP(E51,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>35</v>
       </c>
-      <c r="H51" s="3" t="str">
+      <c r="G51" s="3">
+        <v>24</v>
+      </c>
+      <c r="H51" s="3">
         <f>IF(G51="","",IF(G51="DNS",0,IF(G51="DQ",0,IF(G51="DNF",1,IF(AND(ISNUMBER(G51),G51&gt;59),1,_xlfn.XLOOKUP(G51,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>36</v>
       </c>
       <c r="J51" s="3" t="str">
         <f>IF(I51="","",IF(I51="DNS",0,IF(I51="DQ",0,IF(I51="DNF",1,IF(AND(ISNUMBER(I51),I51&gt;59),1,_xlfn.XLOOKUP(I51,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -5724,7 +5881,7 @@
       </c>
       <c r="Q51" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>35</v>
+        <v>71</v>
       </c>
       <c r="R51" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -5732,7 +5889,7 @@
       </c>
       <c r="S51" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>35</v>
+        <v>71</v>
       </c>
     </row>
     <row r="52" spans="1:19" x14ac:dyDescent="0.4">
@@ -5755,9 +5912,12 @@
         <f>IF(E52="","",IF(E52="DNS",0,IF(E52="DQ",0,IF(E52="DNF",1,IF(AND(ISNUMBER(E52),E52&gt;59),1,_xlfn.XLOOKUP(E52,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>34</v>
       </c>
-      <c r="H52" s="3" t="str">
+      <c r="G52" s="3">
+        <v>32</v>
+      </c>
+      <c r="H52" s="3">
         <f>IF(G52="","",IF(G52="DNS",0,IF(G52="DQ",0,IF(G52="DNF",1,IF(AND(ISNUMBER(G52),G52&gt;59),1,_xlfn.XLOOKUP(G52,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>28</v>
       </c>
       <c r="J52" s="3" t="str">
         <f>IF(I52="","",IF(I52="DNS",0,IF(I52="DQ",0,IF(I52="DNF",1,IF(AND(ISNUMBER(I52),I52&gt;59),1,_xlfn.XLOOKUP(I52,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -5777,15 +5937,15 @@
       </c>
       <c r="Q52" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>34</v>
+        <v>62</v>
       </c>
       <c r="R52" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="S52" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>34</v>
+        <v>62</v>
       </c>
     </row>
     <row r="53" spans="1:19" x14ac:dyDescent="0.4">
@@ -5808,9 +5968,12 @@
         <f>IF(E53="","",IF(E53="DNS",0,IF(E53="DQ",0,IF(E53="DNF",1,IF(AND(ISNUMBER(E53),E53&gt;59),1,_xlfn.XLOOKUP(E53,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>0</v>
       </c>
-      <c r="H53" s="3" t="str">
+      <c r="G53" s="3">
+        <v>26</v>
+      </c>
+      <c r="H53" s="3">
         <f>IF(G53="","",IF(G53="DNS",0,IF(G53="DQ",0,IF(G53="DNF",1,IF(AND(ISNUMBER(G53),G53&gt;59),1,_xlfn.XLOOKUP(G53,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>34</v>
       </c>
       <c r="J53" s="3" t="str">
         <f>IF(I53="","",IF(I53="DNS",0,IF(I53="DQ",0,IF(I53="DNF",1,IF(AND(ISNUMBER(I53),I53&gt;59),1,_xlfn.XLOOKUP(I53,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -5830,7 +5993,7 @@
       </c>
       <c r="Q53" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="R53" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -5838,7 +6001,7 @@
       </c>
       <c r="S53" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>34</v>
       </c>
     </row>
     <row r="54" spans="1:19" x14ac:dyDescent="0.4">
@@ -5861,9 +6024,12 @@
         <f>IF(E54="","",IF(E54="DNS",0,IF(E54="DQ",0,IF(E54="DNF",1,IF(AND(ISNUMBER(E54),E54&gt;59),1,_xlfn.XLOOKUP(E54,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>0</v>
       </c>
-      <c r="H54" s="3" t="str">
+      <c r="G54" s="3">
+        <v>47</v>
+      </c>
+      <c r="H54" s="3">
         <f>IF(G54="","",IF(G54="DNS",0,IF(G54="DQ",0,IF(G54="DNF",1,IF(AND(ISNUMBER(G54),G54&gt;59),1,_xlfn.XLOOKUP(G54,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>13</v>
       </c>
       <c r="J54" s="3" t="str">
         <f>IF(I54="","",IF(I54="DNS",0,IF(I54="DQ",0,IF(I54="DNF",1,IF(AND(ISNUMBER(I54),I54&gt;59),1,_xlfn.XLOOKUP(I54,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -5883,7 +6049,7 @@
       </c>
       <c r="Q54" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="R54" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -5891,7 +6057,7 @@
       </c>
       <c r="S54" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="55" spans="1:19" x14ac:dyDescent="0.4">
@@ -5914,9 +6080,12 @@
         <f>IF(E55="","",IF(E55="DNS",0,IF(E55="DQ",0,IF(E55="DNF",1,IF(AND(ISNUMBER(E55),E55&gt;59),1,_xlfn.XLOOKUP(E55,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>21</v>
       </c>
-      <c r="H55" s="3" t="str">
+      <c r="G55" s="3">
+        <v>45</v>
+      </c>
+      <c r="H55" s="3">
         <f>IF(G55="","",IF(G55="DNS",0,IF(G55="DQ",0,IF(G55="DNF",1,IF(AND(ISNUMBER(G55),G55&gt;59),1,_xlfn.XLOOKUP(G55,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>15</v>
       </c>
       <c r="J55" s="3" t="str">
         <f>IF(I55="","",IF(I55="DNS",0,IF(I55="DQ",0,IF(I55="DNF",1,IF(AND(ISNUMBER(I55),I55&gt;59),1,_xlfn.XLOOKUP(I55,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -5936,15 +6105,15 @@
       </c>
       <c r="Q55" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="R55" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="S55" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>21</v>
+        <v>36</v>
       </c>
     </row>
     <row r="56" spans="1:19" x14ac:dyDescent="0.4">
@@ -5967,9 +6136,12 @@
         <f>IF(E56="","",IF(E56="DNS",0,IF(E56="DQ",0,IF(E56="DNF",1,IF(AND(ISNUMBER(E56),E56&gt;59),1,_xlfn.XLOOKUP(E56,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>0</v>
       </c>
-      <c r="H56" s="3" t="str">
+      <c r="G56" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="H56" s="3">
         <f>IF(G56="","",IF(G56="DNS",0,IF(G56="DQ",0,IF(G56="DNF",1,IF(AND(ISNUMBER(G56),G56&gt;59),1,_xlfn.XLOOKUP(G56,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J56" s="3" t="str">
         <f>IF(I56="","",IF(I56="DNS",0,IF(I56="DQ",0,IF(I56="DNF",1,IF(AND(ISNUMBER(I56),I56&gt;59),1,_xlfn.XLOOKUP(I56,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -6020,9 +6192,12 @@
         <f>IF(E57="","",IF(E57="DNS",0,IF(E57="DQ",0,IF(E57="DNF",1,IF(AND(ISNUMBER(E57),E57&gt;59),1,_xlfn.XLOOKUP(E57,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>49</v>
       </c>
-      <c r="H57" s="3" t="str">
+      <c r="G57" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="H57" s="3">
         <f>IF(G57="","",IF(G57="DNS",0,IF(G57="DQ",0,IF(G57="DNF",1,IF(AND(ISNUMBER(G57),G57&gt;59),1,_xlfn.XLOOKUP(G57,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J57" s="3" t="str">
         <f>IF(I57="","",IF(I57="DNS",0,IF(I57="DQ",0,IF(I57="DNF",1,IF(AND(ISNUMBER(I57),I57&gt;59),1,_xlfn.XLOOKUP(I57,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -6046,7 +6221,7 @@
       </c>
       <c r="R57" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="S57" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
@@ -6073,9 +6248,12 @@
         <f>IF(E58="","",IF(E58="DNS",0,IF(E58="DQ",0,IF(E58="DNF",1,IF(AND(ISNUMBER(E58),E58&gt;59),1,_xlfn.XLOOKUP(E58,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>17</v>
       </c>
-      <c r="H58" s="3" t="str">
+      <c r="G58" s="3">
+        <v>33</v>
+      </c>
+      <c r="H58" s="3">
         <f>IF(G58="","",IF(G58="DNS",0,IF(G58="DQ",0,IF(G58="DNF",1,IF(AND(ISNUMBER(G58),G58&gt;59),1,_xlfn.XLOOKUP(G58,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>27</v>
       </c>
       <c r="J58" s="3" t="str">
         <f>IF(I58="","",IF(I58="DNS",0,IF(I58="DQ",0,IF(I58="DNF",1,IF(AND(ISNUMBER(I58),I58&gt;59),1,_xlfn.XLOOKUP(I58,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -6095,7 +6273,7 @@
       </c>
       <c r="Q58" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="R58" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -6103,7 +6281,7 @@
       </c>
       <c r="S58" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="59" spans="1:19" x14ac:dyDescent="0.4">
@@ -6126,9 +6304,12 @@
         <f>IF(E59="","",IF(E59="DNS",0,IF(E59="DQ",0,IF(E59="DNF",1,IF(AND(ISNUMBER(E59),E59&gt;59),1,_xlfn.XLOOKUP(E59,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>0</v>
       </c>
-      <c r="H59" s="3" t="str">
+      <c r="G59" s="3">
+        <v>44</v>
+      </c>
+      <c r="H59" s="3">
         <f>IF(G59="","",IF(G59="DNS",0,IF(G59="DQ",0,IF(G59="DNF",1,IF(AND(ISNUMBER(G59),G59&gt;59),1,_xlfn.XLOOKUP(G59,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>16</v>
       </c>
       <c r="J59" s="3" t="str">
         <f>IF(I59="","",IF(I59="DNS",0,IF(I59="DQ",0,IF(I59="DNF",1,IF(AND(ISNUMBER(I59),I59&gt;59),1,_xlfn.XLOOKUP(I59,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -6148,7 +6329,7 @@
       </c>
       <c r="Q59" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="R59" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -6156,7 +6337,7 @@
       </c>
       <c r="S59" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>16</v>
       </c>
     </row>
     <row r="60" spans="1:19" x14ac:dyDescent="0.4">
@@ -6179,9 +6360,12 @@
         <f>IF(E60="","",IF(E60="DNS",0,IF(E60="DQ",0,IF(E60="DNF",1,IF(AND(ISNUMBER(E60),E60&gt;59),1,_xlfn.XLOOKUP(E60,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>0</v>
       </c>
-      <c r="H60" s="3" t="str">
+      <c r="G60" s="3">
+        <v>15</v>
+      </c>
+      <c r="H60" s="3">
         <f>IF(G60="","",IF(G60="DNS",0,IF(G60="DQ",0,IF(G60="DNF",1,IF(AND(ISNUMBER(G60),G60&gt;59),1,_xlfn.XLOOKUP(G60,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>45</v>
       </c>
       <c r="J60" s="3" t="str">
         <f>IF(I60="","",IF(I60="DNS",0,IF(I60="DQ",0,IF(I60="DNF",1,IF(AND(ISNUMBER(I60),I60&gt;59),1,_xlfn.XLOOKUP(I60,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -6201,7 +6385,7 @@
       </c>
       <c r="Q60" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="R60" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -6209,7 +6393,7 @@
       </c>
       <c r="S60" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>45</v>
       </c>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.4">
@@ -6232,9 +6416,12 @@
         <f>IF(E61="","",IF(E61="DNS",0,IF(E61="DQ",0,IF(E61="DNF",1,IF(AND(ISNUMBER(E61),E61&gt;59),1,_xlfn.XLOOKUP(E61,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>0</v>
       </c>
-      <c r="H61" s="3" t="str">
+      <c r="G61" s="3">
+        <v>48</v>
+      </c>
+      <c r="H61" s="3">
         <f>IF(G61="","",IF(G61="DNS",0,IF(G61="DQ",0,IF(G61="DNF",1,IF(AND(ISNUMBER(G61),G61&gt;59),1,_xlfn.XLOOKUP(G61,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>12</v>
       </c>
       <c r="J61" s="3" t="str">
         <f>IF(I61="","",IF(I61="DNS",0,IF(I61="DQ",0,IF(I61="DNF",1,IF(AND(ISNUMBER(I61),I61&gt;59),1,_xlfn.XLOOKUP(I61,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -6254,7 +6441,7 @@
       </c>
       <c r="Q61" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="R61" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -6262,7 +6449,7 @@
       </c>
       <c r="S61" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.4">
@@ -6285,9 +6472,12 @@
         <f>IF(E62="","",IF(E62="DNS",0,IF(E62="DQ",0,IF(E62="DNF",1,IF(AND(ISNUMBER(E62),E62&gt;59),1,_xlfn.XLOOKUP(E62,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>0</v>
       </c>
-      <c r="H62" s="3" t="str">
+      <c r="G62" s="3">
+        <v>37</v>
+      </c>
+      <c r="H62" s="3">
         <f>IF(G62="","",IF(G62="DNS",0,IF(G62="DQ",0,IF(G62="DNF",1,IF(AND(ISNUMBER(G62),G62&gt;59),1,_xlfn.XLOOKUP(G62,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>23</v>
       </c>
       <c r="J62" s="3" t="str">
         <f>IF(I62="","",IF(I62="DNS",0,IF(I62="DQ",0,IF(I62="DNF",1,IF(AND(ISNUMBER(I62),I62&gt;59),1,_xlfn.XLOOKUP(I62,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -6307,7 +6497,7 @@
       </c>
       <c r="Q62" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="R62" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -6315,7 +6505,7 @@
       </c>
       <c r="S62" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="63" spans="1:19" x14ac:dyDescent="0.4">
@@ -6338,9 +6528,12 @@
         <f>IF(E63="","",IF(E63="DNS",0,IF(E63="DQ",0,IF(E63="DNF",1,IF(AND(ISNUMBER(E63),E63&gt;59),1,_xlfn.XLOOKUP(E63,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>0</v>
       </c>
-      <c r="H63" s="3" t="str">
+      <c r="G63" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="H63" s="3">
         <f>IF(G63="","",IF(G63="DNS",0,IF(G63="DQ",0,IF(G63="DNF",1,IF(AND(ISNUMBER(G63),G63&gt;59),1,_xlfn.XLOOKUP(G63,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J63" s="3" t="str">
         <f>IF(I63="","",IF(I63="DNS",0,IF(I63="DQ",0,IF(I63="DNF",1,IF(AND(ISNUMBER(I63),I63&gt;59),1,_xlfn.XLOOKUP(I63,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -6391,9 +6584,12 @@
         <f>IF(E64="","",IF(E64="DNS",0,IF(E64="DQ",0,IF(E64="DNF",1,IF(AND(ISNUMBER(E64),E64&gt;59),1,_xlfn.XLOOKUP(E64,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v>0</v>
       </c>
-      <c r="H64" s="3" t="str">
+      <c r="G64" s="3">
+        <v>5</v>
+      </c>
+      <c r="H64" s="3">
         <f>IF(G64="","",IF(G64="DNS",0,IF(G64="DQ",0,IF(G64="DNF",1,IF(AND(ISNUMBER(G64),G64&gt;59),1,_xlfn.XLOOKUP(G64,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>80</v>
       </c>
       <c r="J64" s="3" t="str">
         <f>IF(I64="","",IF(I64="DNS",0,IF(I64="DQ",0,IF(I64="DNF",1,IF(AND(ISNUMBER(I64),I64&gt;59),1,_xlfn.XLOOKUP(I64,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -6413,7 +6609,7 @@
       </c>
       <c r="Q64" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="R64" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
@@ -6421,7 +6617,7 @@
       </c>
       <c r="S64" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="65" spans="1:19" x14ac:dyDescent="0.4">
@@ -6441,9 +6637,12 @@
         <f>IF(E65="","",IF(E65="DNS",0,IF(E65="DQ",0,IF(E65="DNF",1,IF(AND(ISNUMBER(E65),E65&gt;59),1,_xlfn.XLOOKUP(E65,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v/>
       </c>
-      <c r="H65" s="3" t="str">
+      <c r="G65" s="3">
+        <v>18</v>
+      </c>
+      <c r="H65" s="3">
         <f>IF(G65="","",IF(G65="DNS",0,IF(G65="DQ",0,IF(G65="DNF",1,IF(AND(ISNUMBER(G65),G65&gt;59),1,_xlfn.XLOOKUP(G65,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>42</v>
       </c>
       <c r="J65" s="3" t="str">
         <f>IF(I65="","",IF(I65="DNS",0,IF(I65="DQ",0,IF(I65="DNF",1,IF(AND(ISNUMBER(I65),I65&gt;59),1,_xlfn.XLOOKUP(I65,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -6463,15 +6662,15 @@
       </c>
       <c r="Q65" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="R65" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="S65" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>42</v>
       </c>
     </row>
     <row r="66" spans="1:19" x14ac:dyDescent="0.4">
@@ -6491,9 +6690,12 @@
         <f>IF(E66="","",IF(E66="DNS",0,IF(E66="DQ",0,IF(E66="DNF",1,IF(AND(ISNUMBER(E66),E66&gt;59),1,_xlfn.XLOOKUP(E66,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v/>
       </c>
-      <c r="H66" s="3" t="str">
+      <c r="G66" s="3">
+        <v>22</v>
+      </c>
+      <c r="H66" s="3">
         <f>IF(G66="","",IF(G66="DNS",0,IF(G66="DQ",0,IF(G66="DNF",1,IF(AND(ISNUMBER(G66),G66&gt;59),1,_xlfn.XLOOKUP(G66,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>38</v>
       </c>
       <c r="J66" s="3" t="str">
         <f>IF(I66="","",IF(I66="DNS",0,IF(I66="DQ",0,IF(I66="DNF",1,IF(AND(ISNUMBER(I66),I66&gt;59),1,_xlfn.XLOOKUP(I66,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -6513,15 +6715,15 @@
       </c>
       <c r="Q66" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="R66" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="S66" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="67" spans="1:19" x14ac:dyDescent="0.4">
@@ -6541,9 +6743,12 @@
         <f>IF(E67="","",IF(E67="DNS",0,IF(E67="DQ",0,IF(E67="DNF",1,IF(AND(ISNUMBER(E67),E67&gt;59),1,_xlfn.XLOOKUP(E67,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v/>
       </c>
-      <c r="H67" s="3" t="str">
+      <c r="G67" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="H67" s="3">
         <f>IF(G67="","",IF(G67="DNS",0,IF(G67="DQ",0,IF(G67="DNF",1,IF(AND(ISNUMBER(G67),G67&gt;59),1,_xlfn.XLOOKUP(G67,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J67" s="3" t="str">
         <f>IF(I67="","",IF(I67="DNS",0,IF(I67="DQ",0,IF(I67="DNF",1,IF(AND(ISNUMBER(I67),I67&gt;59),1,_xlfn.XLOOKUP(I67,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -6591,9 +6796,12 @@
         <f>IF(E68="","",IF(E68="DNS",0,IF(E68="DQ",0,IF(E68="DNF",1,IF(AND(ISNUMBER(E68),E68&gt;59),1,_xlfn.XLOOKUP(E68,tbl_points[Place],tbl_points[Points],""))))))</f>
         <v/>
       </c>
-      <c r="H68" s="3" t="str">
+      <c r="G68" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="H68" s="3">
         <f>IF(G68="","",IF(G68="DNS",0,IF(G68="DQ",0,IF(G68="DNF",1,IF(AND(ISNUMBER(G68),G68&gt;59),1,_xlfn.XLOOKUP(G68,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J68" s="3" t="str">
         <f>IF(I68="","",IF(I68="DNS",0,IF(I68="DQ",0,IF(I68="DNF",1,IF(AND(ISNUMBER(I68),I68&gt;59),1,_xlfn.XLOOKUP(I68,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -20901,28 +21109,28 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D2:D384">
-    <cfRule type="expression" dxfId="18" priority="1">
+    <cfRule type="expression" dxfId="19" priority="1">
       <formula>$C2="Bant Boys"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="2">
+    <cfRule type="expression" dxfId="18" priority="2">
       <formula>$C2="Bant Girls"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="3">
+    <cfRule type="expression" dxfId="17" priority="3">
       <formula>$C2="Juv Girls"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="4">
+    <cfRule type="expression" dxfId="16" priority="4">
       <formula>$C2="Juv Boys"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="5">
+    <cfRule type="expression" dxfId="15" priority="5">
       <formula>$C2="Jr Girls"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="6">
+    <cfRule type="expression" dxfId="14" priority="6">
       <formula>$C2="Jr Boys"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="7">
+    <cfRule type="expression" dxfId="13" priority="7">
       <formula>$C2="Sr Boys"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="8">
+    <cfRule type="expression" dxfId="12" priority="8">
       <formula>$C2="Sr Girls"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -25901,28 +26109,28 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D2:D384">
-    <cfRule type="expression" dxfId="10" priority="1">
+    <cfRule type="expression" dxfId="11" priority="1">
       <formula>$C2="Bant Boys"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="2">
+    <cfRule type="expression" dxfId="10" priority="2">
       <formula>$C2="Bant Girls"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="3">
+    <cfRule type="expression" dxfId="9" priority="3">
       <formula>$C2="Juv Girls"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="4">
+    <cfRule type="expression" dxfId="8" priority="4">
       <formula>$C2="Juv Boys"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="5">
+    <cfRule type="expression" dxfId="7" priority="5">
       <formula>$C2="Jr Girls"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="6">
+    <cfRule type="expression" dxfId="6" priority="6">
       <formula>$C2="Jr Boys"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="7">
+    <cfRule type="expression" dxfId="5" priority="7">
       <formula>$C2="Sr Boys"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="8">
+    <cfRule type="expression" dxfId="4" priority="8">
       <formula>$C2="Sr Girls"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -26030,7 +26238,7 @@
 )</f>
         <v>265</v>
       </c>
-      <c r="D2" s="3" t="str" cm="1">
+      <c r="D2" s="3" cm="1">
         <f t="array" ref="D2">_xlfn.LET(
 _xlpm.teamDiv,tbl_teampoints[[#This Row],[Division]],
 _xlpm.teamSchool,tbl_teampoints[[#This Row],[School]],
@@ -26061,7 +26269,7 @@
     ""
 )
 )</f>
-        <v/>
+        <v>237</v>
       </c>
       <c r="E2" s="3" t="str" cm="1">
         <f t="array" ref="E2">_xlfn.LET(
@@ -26197,7 +26405,7 @@
       </c>
       <c r="I2" s="3">
         <f>SUM(tbl_teampoints[[#This Row],[Race 1]]:tbl_teampoints[[#This Row],[Race 6]])</f>
-        <v>265</v>
+        <v>502</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.4">
@@ -28130,7 +28338,7 @@
 )</f>
         <v>182</v>
       </c>
-      <c r="D12" s="3" t="str" cm="1">
+      <c r="D12" s="3" cm="1">
         <f t="array" ref="D12">_xlfn.LET(
 _xlpm.teamDiv,tbl_teampoints[[#This Row],[Division]],
 _xlpm.teamSchool,tbl_teampoints[[#This Row],[School]],
@@ -28161,7 +28369,7 @@
     ""
 )
 )</f>
-        <v/>
+        <v>207</v>
       </c>
       <c r="E12" s="3" t="str" cm="1">
         <f t="array" ref="E12">_xlfn.LET(
@@ -28297,7 +28505,7 @@
       </c>
       <c r="I12" s="3">
         <f>SUM(tbl_teampoints[[#This Row],[Race 1]]:tbl_teampoints[[#This Row],[Race 6]])</f>
-        <v>182</v>
+        <v>389</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.4">
@@ -28371,7 +28579,7 @@
     ""
 )
 )</f>
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="E13" s="3" cm="1">
         <f t="array" ref="E13">_xlfn.LET(
@@ -28507,7 +28715,7 @@
       </c>
       <c r="I13" s="3">
         <f>SUM(tbl_teampoints[[#This Row],[Race 1]]:tbl_teampoints[[#This Row],[Race 6]])</f>
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.4">
@@ -28970,7 +29178,7 @@
 )</f>
         <v>0</v>
       </c>
-      <c r="D16" s="3" cm="1">
+      <c r="D16" s="3" t="str" cm="1">
         <f t="array" ref="D16">_xlfn.LET(
 _xlpm.teamDiv,tbl_teampoints[[#This Row],[Division]],
 _xlpm.teamSchool,tbl_teampoints[[#This Row],[School]],
@@ -29001,7 +29209,7 @@
     ""
 )
 )</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E16" s="3" cm="1">
         <f t="array" ref="E16">_xlfn.LET(
@@ -29390,7 +29598,7 @@
 )</f>
         <v>110</v>
       </c>
-      <c r="D18" s="3" cm="1">
+      <c r="D18" s="3" t="str" cm="1">
         <f t="array" ref="D18">_xlfn.LET(
 _xlpm.teamDiv,tbl_teampoints[[#This Row],[Division]],
 _xlpm.teamSchool,tbl_teampoints[[#This Row],[School]],
@@ -29421,7 +29629,7 @@
     ""
 )
 )</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E18" s="3" cm="1">
         <f t="array" ref="E18">_xlfn.LET(
@@ -31311,7 +31519,7 @@
     ""
 )
 )</f>
-        <v>0</v>
+        <v>113</v>
       </c>
       <c r="E27" s="3" cm="1">
         <f t="array" ref="E27">_xlfn.LET(
@@ -31447,7 +31655,7 @@
       </c>
       <c r="I27" s="3">
         <f>SUM(tbl_teampoints[[#This Row],[Race 1]]:tbl_teampoints[[#This Row],[Race 6]])</f>
-        <v>143</v>
+        <v>256</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.4">
@@ -33800,7 +34008,7 @@
 )</f>
         <v/>
       </c>
-      <c r="D39" s="3" t="str" cm="1">
+      <c r="D39" s="3" cm="1">
         <f t="array" ref="D39">_xlfn.LET(
 _xlpm.teamDiv,tbl_teampoints[[#This Row],[Division]],
 _xlpm.teamSchool,tbl_teampoints[[#This Row],[School]],
@@ -33831,7 +34039,7 @@
     ""
 )
 )</f>
-        <v/>
+        <v>62</v>
       </c>
       <c r="E39" s="3" t="str" cm="1">
         <f t="array" ref="E39">_xlfn.LET(
@@ -33967,7 +34175,7 @@
       </c>
       <c r="I39" s="3">
         <f>SUM(tbl_teampoints[[#This Row],[Race 1]]:tbl_teampoints[[#This Row],[Race 6]])</f>
-        <v>0</v>
+        <v>62</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.4">
@@ -34430,7 +34638,7 @@
 )</f>
         <v/>
       </c>
-      <c r="D42" s="3" t="str" cm="1">
+      <c r="D42" s="3" cm="1">
         <f t="array" ref="D42">_xlfn.LET(
 _xlpm.teamDiv,tbl_teampoints[[#This Row],[Division]],
 _xlpm.teamSchool,tbl_teampoints[[#This Row],[School]],
@@ -34461,7 +34669,7 @@
     ""
 )
 )</f>
-        <v/>
+        <v>80</v>
       </c>
       <c r="E42" s="3" t="str" cm="1">
         <f t="array" ref="E42">_xlfn.LET(
@@ -34597,7 +34805,7 @@
       </c>
       <c r="I42" s="3">
         <f>SUM(tbl_teampoints[[#This Row],[Race 1]]:tbl_teampoints[[#This Row],[Race 6]])</f>
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
Fix rider records and team points in results data
Adjust competitor entries across JSON results and update the master spreadsheet. Reconciles name/plate swaps, DNS placements, R1 places/points and point totals for multiple riders (e.g. Jivcko Elvir Sheilds, Felix Carr, Remy Zurbuchen, Marcelo Alcocer Tremari, William Lucas, Ryan Pasha and others). Propagates these fixes into school_results.json and race_results.json, and corrects Handsworth's Race1/team total in team_results.json. Also updates the binary results_2026_master.xlsx to reflect the changes.
</commit_message>
<xml_diff>
--- a/results_2026_master.xlsx
+++ b/results_2026_master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\19247\Documents\codemathbike\codemathbike_bike\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8BFDCEDB-1352-44F5-BA39-1F6B49ED6518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{868182DF-9306-4A6D-B30D-3B6CBBE0220C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1640" yWindow="-20680" windowWidth="28520" windowHeight="18810" activeTab="2" xr2:uid="{E4CCCC36-747C-4C6A-A938-400850181E6F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{E4CCCC36-747C-4C6A-A938-400850181E6F}"/>
   </bookViews>
   <sheets>
     <sheet name="Rosters - notes" sheetId="11" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2496" uniqueCount="426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2497" uniqueCount="426">
   <si>
     <t>Divisions</t>
   </si>
@@ -1857,10 +1857,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{0A7F75BD-58F6-4493-BFAC-CEF3E5A7D6A6}" name="tbl_individual3" displayName="tbl_individual3" ref="A1:E354" totalsRowShown="0" headerRowDxfId="43">
   <autoFilter ref="A1:E354" xr:uid="{4732A653-9976-4BC3-B1BB-3377C0BE5451}">
@@ -1900,11 +1896,11 @@
   <autoFilter ref="A1:S353" xr:uid="{4732A653-9976-4BC3-B1BB-3377C0BE5451}">
     <filterColumn colId="2">
       <filters>
-        <filter val="Juv Boys"/>
+        <filter val="Bant Boys"/>
       </filters>
     </filterColumn>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:S350">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A23:S352">
     <sortCondition ref="E1:E353"/>
   </sortState>
   <tableColumns count="19">
@@ -8439,7 +8435,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>77</v>
       </c>
@@ -8492,7 +8488,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>187</v>
       </c>
@@ -8545,7 +8541,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>73</v>
       </c>
@@ -8598,7 +8594,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>159</v>
       </c>
@@ -8651,7 +8647,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>296</v>
       </c>
@@ -8704,7 +8700,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>291</v>
       </c>
@@ -8757,7 +8753,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>292</v>
       </c>
@@ -8810,7 +8806,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>238</v>
       </c>
@@ -8863,7 +8859,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>250</v>
       </c>
@@ -8916,7 +8912,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>71</v>
       </c>
@@ -8969,7 +8965,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>70</v>
       </c>
@@ -9393,25 +9389,25 @@
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
-        <v>57</v>
+        <v>170</v>
       </c>
       <c r="B23" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="C23" t="s">
         <v>7</v>
       </c>
       <c r="D23" s="3">
-        <v>8147</v>
+        <v>837</v>
       </c>
       <c r="E23" s="3">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="F23" s="3">
         <f>IF(E23="","",IF(E23="DNS",0,IF(E23="DQ",0,IF(E23="DNF",1,IF(AND(ISNUMBER(E23),E23&gt;59),1,_xlfn.XLOOKUP(E23,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>37</v>
+        <v>100</v>
       </c>
       <c r="H23" s="3" t="str">
         <f>IF(G23="","",IF(G23="DNS",0,IF(G23="DQ",0,IF(G23="DNF",1,IF(AND(ISNUMBER(G23),G23&gt;59),1,_xlfn.XLOOKUP(G23,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -9435,15 +9431,15 @@
       </c>
       <c r="Q23" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>37</v>
+        <v>100</v>
       </c>
       <c r="R23" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>37</v>
+        <v>100</v>
       </c>
       <c r="S23" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>37</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -9552,25 +9548,25 @@
         <v>53</v>
       </c>
     </row>
-    <row r="26" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
-        <v>54</v>
+        <v>171</v>
       </c>
       <c r="B26" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="C26" t="s">
         <v>7</v>
       </c>
       <c r="D26" s="3">
-        <v>8049</v>
+        <v>838</v>
       </c>
       <c r="E26" s="3">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="F26" s="3">
         <f>IF(E26="","",IF(E26="DNS",0,IF(E26="DQ",0,IF(E26="DNF",1,IF(AND(ISNUMBER(E26),E26&gt;59),1,_xlfn.XLOOKUP(E26,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>35</v>
+        <v>95</v>
       </c>
       <c r="H26" s="3" t="str">
         <f>IF(G26="","",IF(G26="DNS",0,IF(G26="DQ",0,IF(G26="DNF",1,IF(AND(ISNUMBER(G26),G26&gt;59),1,_xlfn.XLOOKUP(G26,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -9594,15 +9590,15 @@
       </c>
       <c r="Q26" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>35</v>
+        <v>95</v>
       </c>
       <c r="R26" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>35</v>
+        <v>95</v>
       </c>
       <c r="S26" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>35</v>
+        <v>95</v>
       </c>
     </row>
     <row r="27" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -10135,25 +10131,25 @@
         <v>22</v>
       </c>
     </row>
-    <row r="37" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
-        <v>61</v>
+        <v>140</v>
       </c>
       <c r="B37" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C37" t="s">
         <v>7</v>
       </c>
       <c r="D37" s="3">
-        <v>8185</v>
-      </c>
-      <c r="E37" s="3" t="s">
-        <v>415</v>
+        <v>8196</v>
+      </c>
+      <c r="E37" s="3">
+        <v>3</v>
       </c>
       <c r="F37" s="3">
         <f>IF(E37="","",IF(E37="DNS",0,IF(E37="DQ",0,IF(E37="DNF",1,IF(AND(ISNUMBER(E37),E37&gt;59),1,_xlfn.XLOOKUP(E37,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>1</v>
+        <v>90</v>
       </c>
       <c r="H37" s="3" t="str">
         <f>IF(G37="","",IF(G37="DNS",0,IF(G37="DQ",0,IF(G37="DNF",1,IF(AND(ISNUMBER(G37),G37&gt;59),1,_xlfn.XLOOKUP(G37,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -10177,36 +10173,36 @@
       </c>
       <c r="Q37" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>1</v>
+        <v>90</v>
       </c>
       <c r="R37" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>1</v>
+        <v>90</v>
       </c>
       <c r="S37" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="38" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
-        <v>53</v>
+        <v>143</v>
       </c>
       <c r="B38" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C38" t="s">
         <v>7</v>
       </c>
       <c r="D38" s="3">
-        <v>8010</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>416</v>
+        <v>8198</v>
+      </c>
+      <c r="E38" s="3">
+        <v>3</v>
       </c>
       <c r="F38" s="3">
         <f>IF(E38="","",IF(E38="DNS",0,IF(E38="DQ",0,IF(E38="DNF",1,IF(AND(ISNUMBER(E38),E38&gt;59),1,_xlfn.XLOOKUP(E38,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="H38" s="3" t="str">
         <f>IF(G38="","",IF(G38="DNS",0,IF(G38="DQ",0,IF(G38="DNF",1,IF(AND(ISNUMBER(G38),G38&gt;59),1,_xlfn.XLOOKUP(G38,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -10230,36 +10226,36 @@
       </c>
       <c r="Q38" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="R38" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="S38" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="39" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
-        <v>55</v>
+        <v>414</v>
       </c>
       <c r="B39" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="C39" t="s">
         <v>7</v>
       </c>
       <c r="D39" s="3">
-        <v>8086</v>
-      </c>
-      <c r="E39" s="3" t="s">
-        <v>416</v>
+        <v>839</v>
+      </c>
+      <c r="E39" s="3">
+        <v>4</v>
       </c>
       <c r="F39" s="3">
         <f>IF(E39="","",IF(E39="DNS",0,IF(E39="DQ",0,IF(E39="DNF",1,IF(AND(ISNUMBER(E39),E39&gt;59),1,_xlfn.XLOOKUP(E39,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="H39" s="3" t="str">
         <f>IF(G39="","",IF(G39="DNS",0,IF(G39="DQ",0,IF(G39="DNF",1,IF(AND(ISNUMBER(G39),G39&gt;59),1,_xlfn.XLOOKUP(G39,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -10283,15 +10279,15 @@
       </c>
       <c r="Q39" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="R39" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="S39" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>85</v>
       </c>
     </row>
     <row r="40" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -10877,25 +10873,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
-        <v>56</v>
+        <v>245</v>
       </c>
       <c r="B51" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C51" t="s">
         <v>7</v>
       </c>
       <c r="D51" s="3">
-        <v>8140</v>
-      </c>
-      <c r="E51" s="3" t="s">
-        <v>416</v>
+        <v>816</v>
+      </c>
+      <c r="E51" s="3">
+        <v>5</v>
       </c>
       <c r="F51" s="3">
         <f>IF(E51="","",IF(E51="DNS",0,IF(E51="DQ",0,IF(E51="DNF",1,IF(AND(ISNUMBER(E51),E51&gt;59),1,_xlfn.XLOOKUP(E51,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="H51" s="3" t="str">
         <f>IF(G51="","",IF(G51="DNS",0,IF(G51="DQ",0,IF(G51="DNF",1,IF(AND(ISNUMBER(G51),G51&gt;59),1,_xlfn.XLOOKUP(G51,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -10919,36 +10915,36 @@
       </c>
       <c r="Q51" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="R51" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="S51" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="52" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
-        <v>58</v>
+        <v>351</v>
       </c>
       <c r="B52" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="C52" t="s">
         <v>7</v>
       </c>
       <c r="D52" s="3">
-        <v>8154</v>
-      </c>
-      <c r="E52" s="3" t="s">
-        <v>416</v>
+        <v>831</v>
+      </c>
+      <c r="E52" s="3">
+        <v>6</v>
       </c>
       <c r="F52" s="3">
         <f>IF(E52="","",IF(E52="DNS",0,IF(E52="DQ",0,IF(E52="DNF",1,IF(AND(ISNUMBER(E52),E52&gt;59),1,_xlfn.XLOOKUP(E52,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="H52" s="3" t="str">
         <f>IF(G52="","",IF(G52="DNS",0,IF(G52="DQ",0,IF(G52="DNF",1,IF(AND(ISNUMBER(G52),G52&gt;59),1,_xlfn.XLOOKUP(G52,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -10972,36 +10968,36 @@
       </c>
       <c r="Q52" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="R52" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="S52" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="53" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
-        <v>59</v>
+        <v>352</v>
       </c>
       <c r="B53" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="C53" t="s">
         <v>7</v>
       </c>
       <c r="D53" s="3">
-        <v>8177</v>
-      </c>
-      <c r="E53" s="3" t="s">
-        <v>416</v>
+        <v>832</v>
+      </c>
+      <c r="E53" s="3">
+        <v>7</v>
       </c>
       <c r="F53" s="3">
         <f>IF(E53="","",IF(E53="DNS",0,IF(E53="DQ",0,IF(E53="DNF",1,IF(AND(ISNUMBER(E53),E53&gt;59),1,_xlfn.XLOOKUP(E53,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="H53" s="3" t="str">
         <f>IF(G53="","",IF(G53="DNS",0,IF(G53="DQ",0,IF(G53="DNF",1,IF(AND(ISNUMBER(G53),G53&gt;59),1,_xlfn.XLOOKUP(G53,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -11025,36 +11021,36 @@
       </c>
       <c r="Q53" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="R53" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="S53" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="54" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
-        <v>60</v>
+        <v>155</v>
       </c>
       <c r="B54" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C54" t="s">
         <v>7</v>
       </c>
       <c r="D54" s="3">
-        <v>8181</v>
-      </c>
-      <c r="E54" s="3" t="s">
-        <v>416</v>
+        <v>804</v>
+      </c>
+      <c r="E54" s="3">
+        <v>8</v>
       </c>
       <c r="F54" s="3">
         <f>IF(E54="","",IF(E54="DNS",0,IF(E54="DQ",0,IF(E54="DNF",1,IF(AND(ISNUMBER(E54),E54&gt;59),1,_xlfn.XLOOKUP(E54,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="H54" s="3" t="str">
         <f>IF(G54="","",IF(G54="DNS",0,IF(G54="DQ",0,IF(G54="DNF",1,IF(AND(ISNUMBER(G54),G54&gt;59),1,_xlfn.XLOOKUP(G54,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -11078,36 +11074,36 @@
       </c>
       <c r="Q54" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="R54" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="S54" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="55" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
-        <v>62</v>
+        <v>408</v>
       </c>
       <c r="B55" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C55" t="s">
         <v>7</v>
       </c>
       <c r="D55" s="3">
-        <v>8186</v>
-      </c>
-      <c r="E55" s="3" t="s">
-        <v>416</v>
+        <v>8009</v>
+      </c>
+      <c r="E55" s="3">
+        <v>9</v>
       </c>
       <c r="F55" s="3">
         <f>IF(E55="","",IF(E55="DNS",0,IF(E55="DQ",0,IF(E55="DNF",1,IF(AND(ISNUMBER(E55),E55&gt;59),1,_xlfn.XLOOKUP(E55,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="H55" s="3" t="str">
         <f>IF(G55="","",IF(G55="DNS",0,IF(G55="DQ",0,IF(G55="DNF",1,IF(AND(ISNUMBER(G55),G55&gt;59),1,_xlfn.XLOOKUP(G55,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -11131,15 +11127,15 @@
       </c>
       <c r="Q55" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="R55" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="S55" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="56" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -11195,7 +11191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
         <v>418</v>
       </c>
@@ -11301,7 +11297,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A59" t="s">
         <v>69</v>
       </c>
@@ -11354,25 +11350,25 @@
         <v>49</v>
       </c>
     </row>
-    <row r="60" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A60" t="s">
-        <v>103</v>
+        <v>313</v>
       </c>
       <c r="B60" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="C60" t="s">
         <v>7</v>
       </c>
       <c r="D60" s="3">
-        <v>8189</v>
+        <v>824</v>
       </c>
       <c r="E60" s="3">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="F60" s="3">
         <f>IF(E60="","",IF(E60="DNS",0,IF(E60="DQ",0,IF(E60="DNF",1,IF(AND(ISNUMBER(E60),E60&gt;59),1,_xlfn.XLOOKUP(E60,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="H60" s="3" t="str">
         <f>IF(G60="","",IF(G60="DNS",0,IF(G60="DQ",0,IF(G60="DNF",1,IF(AND(ISNUMBER(G60),G60&gt;59),1,_xlfn.XLOOKUP(G60,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -11396,15 +11392,15 @@
       </c>
       <c r="Q60" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="R60" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="S60" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>27</v>
+        <v>55</v>
       </c>
     </row>
     <row r="61" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -11725,25 +11721,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A67" t="s">
-        <v>104</v>
+        <v>142</v>
       </c>
       <c r="B67" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C67" t="s">
         <v>7</v>
       </c>
       <c r="D67" s="3">
-        <v>8190</v>
-      </c>
-      <c r="E67" s="3" t="s">
-        <v>416</v>
+        <v>8197</v>
+      </c>
+      <c r="E67" s="3">
+        <v>11</v>
       </c>
       <c r="F67" s="3">
         <f>IF(E67="","",IF(E67="DNS",0,IF(E67="DQ",0,IF(E67="DNF",1,IF(AND(ISNUMBER(E67),E67&gt;59),1,_xlfn.XLOOKUP(E67,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="H67" s="3" t="str">
         <f>IF(G67="","",IF(G67="DNS",0,IF(G67="DQ",0,IF(G67="DNF",1,IF(AND(ISNUMBER(G67),G67&gt;59),1,_xlfn.XLOOKUP(G67,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -11767,15 +11763,15 @@
       </c>
       <c r="Q67" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="R67" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="S67" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>53</v>
       </c>
     </row>
     <row r="68" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -11831,25 +11827,25 @@
         <v>90</v>
       </c>
     </row>
-    <row r="69" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A69" t="s">
-        <v>113</v>
+        <v>305</v>
       </c>
       <c r="B69" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="C69" t="s">
         <v>7</v>
       </c>
       <c r="D69" s="3">
-        <v>8191</v>
+        <v>823</v>
       </c>
       <c r="E69" s="3">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F69" s="3">
         <f>IF(E69="","",IF(E69="DNS",0,IF(E69="DQ",0,IF(E69="DNF",1,IF(AND(ISNUMBER(E69),E69&gt;59),1,_xlfn.XLOOKUP(E69,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="H69" s="3" t="str">
         <f>IF(G69="","",IF(G69="DNS",0,IF(G69="DQ",0,IF(G69="DNF",1,IF(AND(ISNUMBER(G69),G69&gt;59),1,_xlfn.XLOOKUP(G69,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -11873,36 +11869,36 @@
       </c>
       <c r="Q69" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="R69" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="S69" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="70" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="70" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A70" t="s">
-        <v>114</v>
+        <v>314</v>
       </c>
       <c r="B70" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="C70" t="s">
         <v>7</v>
       </c>
       <c r="D70" s="3">
-        <v>8192</v>
+        <v>825</v>
       </c>
       <c r="E70" s="3">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="F70" s="3">
         <f>IF(E70="","",IF(E70="DNS",0,IF(E70="DQ",0,IF(E70="DNF",1,IF(AND(ISNUMBER(E70),E70&gt;59),1,_xlfn.XLOOKUP(E70,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="H70" s="3" t="str">
         <f>IF(G70="","",IF(G70="DNS",0,IF(G70="DQ",0,IF(G70="DNF",1,IF(AND(ISNUMBER(G70),G70&gt;59),1,_xlfn.XLOOKUP(G70,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -11926,15 +11922,15 @@
       </c>
       <c r="Q70" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="R70" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="S70" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>31</v>
+        <v>49</v>
       </c>
     </row>
     <row r="71" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -12467,7 +12463,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A81" t="s">
         <v>337</v>
       </c>
@@ -12520,7 +12516,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A82" t="s">
         <v>72</v>
       </c>
@@ -12944,25 +12940,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A90" t="s">
-        <v>122</v>
+        <v>246</v>
       </c>
       <c r="B90" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="C90" t="s">
         <v>7</v>
       </c>
       <c r="D90" s="3">
-        <v>8193</v>
-      </c>
-      <c r="E90" s="3" t="s">
-        <v>416</v>
+        <v>817</v>
+      </c>
+      <c r="E90" s="3">
+        <v>14</v>
       </c>
       <c r="F90" s="3">
         <f>IF(E90="","",IF(E90="DNS",0,IF(E90="DQ",0,IF(E90="DNF",1,IF(AND(ISNUMBER(E90),E90&gt;59),1,_xlfn.XLOOKUP(E90,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="H90" s="3" t="str">
         <f>IF(G90="","",IF(G90="DNS",0,IF(G90="DQ",0,IF(G90="DNF",1,IF(AND(ISNUMBER(G90),G90&gt;59),1,_xlfn.XLOOKUP(G90,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -12986,36 +12982,36 @@
       </c>
       <c r="Q90" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="R90" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="S90" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="91" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="91" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A91" t="s">
-        <v>123</v>
+        <v>356</v>
       </c>
       <c r="B91" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="C91" t="s">
         <v>7</v>
       </c>
       <c r="D91" s="3">
-        <v>8194</v>
-      </c>
-      <c r="E91" s="3" t="s">
-        <v>416</v>
+        <v>833</v>
+      </c>
+      <c r="E91" s="3">
+        <v>15</v>
       </c>
       <c r="F91" s="3">
         <f>IF(E91="","",IF(E91="DNS",0,IF(E91="DQ",0,IF(E91="DNF",1,IF(AND(ISNUMBER(E91),E91&gt;59),1,_xlfn.XLOOKUP(E91,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="H91" s="3" t="str">
         <f>IF(G91="","",IF(G91="DNS",0,IF(G91="DQ",0,IF(G91="DNF",1,IF(AND(ISNUMBER(G91),G91&gt;59),1,_xlfn.XLOOKUP(G91,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -13039,15 +13035,15 @@
       </c>
       <c r="Q91" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="R91" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="S91" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>45</v>
       </c>
     </row>
     <row r="92" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -13156,25 +13152,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="94" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A94" t="s">
-        <v>140</v>
+        <v>331</v>
       </c>
       <c r="B94" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="C94" t="s">
         <v>7</v>
       </c>
       <c r="D94" s="3">
-        <v>8196</v>
+        <v>826</v>
       </c>
       <c r="E94" s="3">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="F94" s="3">
         <f>IF(E94="","",IF(E94="DNS",0,IF(E94="DQ",0,IF(E94="DNF",1,IF(AND(ISNUMBER(E94),E94&gt;59),1,_xlfn.XLOOKUP(E94,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>90</v>
+        <v>44</v>
       </c>
       <c r="H94" s="3" t="str">
         <f>IF(G94="","",IF(G94="DNS",0,IF(G94="DQ",0,IF(G94="DNF",1,IF(AND(ISNUMBER(G94),G94&gt;59),1,_xlfn.XLOOKUP(G94,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -13198,15 +13194,15 @@
       </c>
       <c r="Q94" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>90</v>
+        <v>44</v>
       </c>
       <c r="R94" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>90</v>
+        <v>44</v>
       </c>
       <c r="S94" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>90</v>
+        <v>44</v>
       </c>
     </row>
     <row r="95" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -13315,25 +13311,25 @@
         <v>34</v>
       </c>
     </row>
-    <row r="97" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="97" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A97" t="s">
-        <v>139</v>
+        <v>184</v>
       </c>
       <c r="B97" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C97" t="s">
         <v>7</v>
       </c>
       <c r="D97" s="3">
-        <v>8195</v>
-      </c>
-      <c r="E97" s="3" t="s">
-        <v>416</v>
+        <v>810</v>
+      </c>
+      <c r="E97" s="3">
+        <v>17</v>
       </c>
       <c r="F97" s="3">
         <f>IF(E97="","",IF(E97="DNS",0,IF(E97="DQ",0,IF(E97="DNF",1,IF(AND(ISNUMBER(E97),E97&gt;59),1,_xlfn.XLOOKUP(E97,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="H97" s="3" t="str">
         <f>IF(G97="","",IF(G97="DNS",0,IF(G97="DQ",0,IF(G97="DNF",1,IF(AND(ISNUMBER(G97),G97&gt;59),1,_xlfn.XLOOKUP(G97,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -13357,36 +13353,36 @@
       </c>
       <c r="Q97" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="R97" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="S97" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="98" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="98" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A98" t="s">
-        <v>143</v>
+        <v>237</v>
       </c>
       <c r="B98" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C98" t="s">
         <v>7</v>
       </c>
       <c r="D98" s="3">
-        <v>8198</v>
+        <v>814</v>
       </c>
       <c r="E98" s="3">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="F98" s="3">
         <f>IF(E98="","",IF(E98="DNS",0,IF(E98="DQ",0,IF(E98="DNF",1,IF(AND(ISNUMBER(E98),E98&gt;59),1,_xlfn.XLOOKUP(E98,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>90</v>
+        <v>42</v>
       </c>
       <c r="H98" s="3" t="str">
         <f>IF(G98="","",IF(G98="DNS",0,IF(G98="DQ",0,IF(G98="DNF",1,IF(AND(ISNUMBER(G98),G98&gt;59),1,_xlfn.XLOOKUP(G98,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -13410,15 +13406,15 @@
       </c>
       <c r="Q98" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>90</v>
+        <v>42</v>
       </c>
       <c r="R98" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>90</v>
+        <v>42</v>
       </c>
       <c r="S98" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>90</v>
+        <v>42</v>
       </c>
     </row>
     <row r="99" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -13474,25 +13470,25 @@
         <v>80</v>
       </c>
     </row>
-    <row r="100" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="100" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A100" t="s">
-        <v>408</v>
+        <v>244</v>
       </c>
       <c r="B100" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C100" t="s">
         <v>7</v>
       </c>
       <c r="D100" s="3">
-        <v>8009</v>
+        <v>815</v>
       </c>
       <c r="E100" s="3">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F100" s="3">
         <f>IF(E100="","",IF(E100="DNS",0,IF(E100="DQ",0,IF(E100="DNF",1,IF(AND(ISNUMBER(E100),E100&gt;59),1,_xlfn.XLOOKUP(E100,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="H100" s="3" t="str">
         <f>IF(G100="","",IF(G100="DNS",0,IF(G100="DQ",0,IF(G100="DNF",1,IF(AND(ISNUMBER(G100),G100&gt;59),1,_xlfn.XLOOKUP(G100,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -13516,36 +13512,36 @@
       </c>
       <c r="Q100" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="R100" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="S100" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>60</v>
-      </c>
-    </row>
-    <row r="101" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="101" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A101" t="s">
-        <v>142</v>
+        <v>302</v>
       </c>
       <c r="B101" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="C101" t="s">
         <v>7</v>
       </c>
       <c r="D101" s="3">
-        <v>8197</v>
+        <v>820</v>
       </c>
       <c r="E101" s="3">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F101" s="3">
         <f>IF(E101="","",IF(E101="DNS",0,IF(E101="DQ",0,IF(E101="DNF",1,IF(AND(ISNUMBER(E101),E101&gt;59),1,_xlfn.XLOOKUP(E101,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="H101" s="3" t="str">
         <f>IF(G101="","",IF(G101="DNS",0,IF(G101="DQ",0,IF(G101="DNF",1,IF(AND(ISNUMBER(G101),G101&gt;59),1,_xlfn.XLOOKUP(G101,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -13569,15 +13565,15 @@
       </c>
       <c r="Q101" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="R101" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="S101" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>53</v>
+        <v>40</v>
       </c>
     </row>
     <row r="102" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -13633,25 +13629,25 @@
         <v>65</v>
       </c>
     </row>
-    <row r="103" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="103" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A103" t="s">
-        <v>145</v>
+        <v>334</v>
       </c>
       <c r="B103" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C103" t="s">
         <v>7</v>
       </c>
       <c r="D103" s="3">
-        <v>800</v>
+        <v>829</v>
       </c>
       <c r="E103" s="3">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F103" s="3">
         <f>IF(E103="","",IF(E103="DNS",0,IF(E103="DQ",0,IF(E103="DNF",1,IF(AND(ISNUMBER(E103),E103&gt;59),1,_xlfn.XLOOKUP(E103,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="H103" s="3" t="str">
         <f>IF(G103="","",IF(G103="DNS",0,IF(G103="DQ",0,IF(G103="DNF",1,IF(AND(ISNUMBER(G103),G103&gt;59),1,_xlfn.XLOOKUP(G103,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -13675,15 +13671,15 @@
       </c>
       <c r="Q103" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="R103" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="S103" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="104" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -13898,25 +13894,25 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="108" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A108" t="s">
-        <v>146</v>
+        <v>113</v>
       </c>
       <c r="B108" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C108" t="s">
         <v>7</v>
       </c>
       <c r="D108" s="3">
-        <v>801</v>
-      </c>
-      <c r="E108" s="3" t="s">
-        <v>416</v>
+        <v>8191</v>
+      </c>
+      <c r="E108" s="3">
+        <v>22</v>
       </c>
       <c r="F108" s="3">
         <f>IF(E108="","",IF(E108="DNS",0,IF(E108="DQ",0,IF(E108="DNF",1,IF(AND(ISNUMBER(E108),E108&gt;59),1,_xlfn.XLOOKUP(E108,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="H108" s="3" t="str">
         <f>IF(G108="","",IF(G108="DNS",0,IF(G108="DQ",0,IF(G108="DNF",1,IF(AND(ISNUMBER(G108),G108&gt;59),1,_xlfn.XLOOKUP(G108,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -13940,36 +13936,36 @@
       </c>
       <c r="Q108" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="R108" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="S108" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="109" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="109" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A109" t="s">
-        <v>144</v>
+        <v>57</v>
       </c>
       <c r="B109" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C109" t="s">
         <v>7</v>
       </c>
       <c r="D109" s="3">
-        <v>8199</v>
-      </c>
-      <c r="E109" s="3" t="s">
-        <v>416</v>
+        <v>8147</v>
+      </c>
+      <c r="E109" s="3">
+        <v>23</v>
       </c>
       <c r="F109" s="3">
         <f>IF(E109="","",IF(E109="DNS",0,IF(E109="DQ",0,IF(E109="DNF",1,IF(AND(ISNUMBER(E109),E109&gt;59),1,_xlfn.XLOOKUP(E109,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="H109" s="3" t="str">
         <f>IF(G109="","",IF(G109="DNS",0,IF(G109="DQ",0,IF(G109="DNF",1,IF(AND(ISNUMBER(G109),G109&gt;59),1,_xlfn.XLOOKUP(G109,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -13993,36 +13989,36 @@
       </c>
       <c r="Q109" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="R109" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="S109" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="110" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="110" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A110" t="s">
-        <v>155</v>
+        <v>303</v>
       </c>
       <c r="B110" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="C110" t="s">
         <v>7</v>
       </c>
       <c r="D110" s="3">
-        <v>804</v>
+        <v>821</v>
       </c>
       <c r="E110" s="3">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="F110" s="3">
         <f>IF(E110="","",IF(E110="DNS",0,IF(E110="DQ",0,IF(E110="DNF",1,IF(AND(ISNUMBER(E110),E110&gt;59),1,_xlfn.XLOOKUP(E110,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="H110" s="3" t="str">
         <f>IF(G110="","",IF(G110="DNS",0,IF(G110="DQ",0,IF(G110="DNF",1,IF(AND(ISNUMBER(G110),G110&gt;59),1,_xlfn.XLOOKUP(G110,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -14046,15 +14042,15 @@
       </c>
       <c r="Q110" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="R110" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="S110" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>65</v>
+        <v>36</v>
       </c>
     </row>
     <row r="111" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -14110,7 +14106,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="112" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="112" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A112" t="s">
         <v>190</v>
       </c>
@@ -14163,7 +14159,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="113" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="113" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A113" t="s">
         <v>353</v>
       </c>
@@ -14216,7 +14212,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="114" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="114" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A114" t="s">
         <v>354</v>
       </c>
@@ -14269,7 +14265,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="115" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="115" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A115" t="s">
         <v>158</v>
       </c>
@@ -14428,25 +14424,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="118" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A118" t="s">
-        <v>154</v>
+        <v>54</v>
       </c>
       <c r="B118" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C118" t="s">
         <v>7</v>
       </c>
       <c r="D118" s="3">
-        <v>803</v>
-      </c>
-      <c r="E118" s="3" t="s">
-        <v>416</v>
+        <v>8049</v>
+      </c>
+      <c r="E118" s="3">
+        <v>25</v>
       </c>
       <c r="F118" s="3">
         <f>IF(E118="","",IF(E118="DNS",0,IF(E118="DQ",0,IF(E118="DNF",1,IF(AND(ISNUMBER(E118),E118&gt;59),1,_xlfn.XLOOKUP(E118,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H118" s="3" t="str">
         <f>IF(G118="","",IF(G118="DNS",0,IF(G118="DQ",0,IF(G118="DNF",1,IF(AND(ISNUMBER(G118),G118&gt;59),1,_xlfn.XLOOKUP(G118,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -14470,36 +14466,36 @@
       </c>
       <c r="Q118" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="R118" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="S118" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="119" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="119" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A119" t="s">
-        <v>170</v>
+        <v>145</v>
       </c>
       <c r="B119" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C119" t="s">
         <v>7</v>
       </c>
       <c r="D119" s="3">
-        <v>837</v>
+        <v>800</v>
       </c>
       <c r="E119" s="3">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="F119" s="3">
         <f>IF(E119="","",IF(E119="DNS",0,IF(E119="DQ",0,IF(E119="DNF",1,IF(AND(ISNUMBER(E119),E119&gt;59),1,_xlfn.XLOOKUP(E119,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>100</v>
+        <v>34</v>
       </c>
       <c r="H119" s="3" t="str">
         <f>IF(G119="","",IF(G119="DNS",0,IF(G119="DQ",0,IF(G119="DNF",1,IF(AND(ISNUMBER(G119),G119&gt;59),1,_xlfn.XLOOKUP(G119,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -14523,36 +14519,36 @@
       </c>
       <c r="Q119" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>100</v>
+        <v>34</v>
       </c>
       <c r="R119" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>100</v>
+        <v>34</v>
       </c>
       <c r="S119" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>100</v>
-      </c>
-    </row>
-    <row r="120" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="120" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A120" t="s">
-        <v>171</v>
+        <v>304</v>
       </c>
       <c r="B120" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="C120" t="s">
         <v>7</v>
       </c>
       <c r="D120" s="3">
-        <v>838</v>
+        <v>822</v>
       </c>
       <c r="E120" s="3">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="F120" s="3">
         <f>IF(E120="","",IF(E120="DNS",0,IF(E120="DQ",0,IF(E120="DNF",1,IF(AND(ISNUMBER(E120),E120&gt;59),1,_xlfn.XLOOKUP(E120,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>95</v>
+        <v>33</v>
       </c>
       <c r="H120" s="3" t="str">
         <f>IF(G120="","",IF(G120="DNS",0,IF(G120="DQ",0,IF(G120="DNF",1,IF(AND(ISNUMBER(G120),G120&gt;59),1,_xlfn.XLOOKUP(G120,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -14576,36 +14572,36 @@
       </c>
       <c r="Q120" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>95</v>
+        <v>33</v>
       </c>
       <c r="R120" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>95</v>
+        <v>33</v>
       </c>
       <c r="S120" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>95</v>
-      </c>
-    </row>
-    <row r="121" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="121" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A121" t="s">
-        <v>414</v>
+        <v>281</v>
       </c>
       <c r="B121" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C121" t="s">
         <v>7</v>
       </c>
       <c r="D121" s="3">
-        <v>839</v>
+        <v>819</v>
       </c>
       <c r="E121" s="3">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="F121" s="3">
         <f>IF(E121="","",IF(E121="DNS",0,IF(E121="DQ",0,IF(E121="DNF",1,IF(AND(ISNUMBER(E121),E121&gt;59),1,_xlfn.XLOOKUP(E121,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>85</v>
+        <v>32</v>
       </c>
       <c r="H121" s="3" t="str">
         <f>IF(G121="","",IF(G121="DNS",0,IF(G121="DQ",0,IF(G121="DNF",1,IF(AND(ISNUMBER(G121),G121&gt;59),1,_xlfn.XLOOKUP(G121,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -14629,15 +14625,15 @@
       </c>
       <c r="Q121" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>85</v>
+        <v>32</v>
       </c>
       <c r="R121" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>85</v>
+        <v>32</v>
       </c>
       <c r="S121" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>85</v>
+        <v>32</v>
       </c>
     </row>
     <row r="122" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -14746,7 +14742,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="124" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="124" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A124" t="s">
         <v>318</v>
       </c>
@@ -14799,7 +14795,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="125" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="125" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A125" t="s">
         <v>293</v>
       </c>
@@ -14852,7 +14848,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="126" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="126" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A126" t="s">
         <v>338</v>
       </c>
@@ -14905,7 +14901,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="127" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="127" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A127" t="s">
         <v>339</v>
       </c>
@@ -15011,25 +15007,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="129" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A129" t="s">
-        <v>172</v>
+        <v>114</v>
       </c>
       <c r="B129" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="C129" t="s">
         <v>7</v>
       </c>
       <c r="D129" s="3">
-        <v>806</v>
+        <v>8192</v>
       </c>
       <c r="E129" s="3">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="F129" s="3">
         <f>IF(E129="","",IF(E129="DNS",0,IF(E129="DQ",0,IF(E129="DNF",1,IF(AND(ISNUMBER(E129),E129&gt;59),1,_xlfn.XLOOKUP(E129,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>75</v>
+        <v>31</v>
       </c>
       <c r="H129" s="3" t="str">
         <f>IF(G129="","",IF(G129="DNS",0,IF(G129="DQ",0,IF(G129="DNF",1,IF(AND(ISNUMBER(G129),G129&gt;59),1,_xlfn.XLOOKUP(G129,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -15053,15 +15049,15 @@
       </c>
       <c r="Q129" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>75</v>
+        <v>31</v>
       </c>
       <c r="R129" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>75</v>
+        <v>31</v>
       </c>
       <c r="S129" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>75</v>
+        <v>31</v>
       </c>
     </row>
     <row r="130" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -15170,25 +15166,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="132" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A132" t="s">
-        <v>173</v>
+        <v>280</v>
       </c>
       <c r="B132" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C132" t="s">
         <v>7</v>
       </c>
       <c r="D132" s="3">
-        <v>807</v>
-      </c>
-      <c r="E132" s="3" t="s">
-        <v>416</v>
+        <v>818</v>
+      </c>
+      <c r="E132" s="3">
+        <v>30</v>
       </c>
       <c r="F132" s="3">
         <f>IF(E132="","",IF(E132="DNS",0,IF(E132="DQ",0,IF(E132="DNF",1,IF(AND(ISNUMBER(E132),E132&gt;59),1,_xlfn.XLOOKUP(E132,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="H132" s="3" t="str">
         <f>IF(G132="","",IF(G132="DNS",0,IF(G132="DQ",0,IF(G132="DNF",1,IF(AND(ISNUMBER(G132),G132&gt;59),1,_xlfn.XLOOKUP(G132,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -15212,36 +15208,36 @@
       </c>
       <c r="Q132" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="R132" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="S132" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="133" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="133" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A133" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="B133" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C133" t="s">
         <v>7</v>
       </c>
       <c r="D133" s="3">
-        <v>808</v>
-      </c>
-      <c r="E133" s="3" t="s">
-        <v>416</v>
+        <v>812</v>
+      </c>
+      <c r="E133" s="3">
+        <v>31</v>
       </c>
       <c r="F133" s="3">
         <f>IF(E133="","",IF(E133="DNS",0,IF(E133="DQ",0,IF(E133="DNF",1,IF(AND(ISNUMBER(E133),E133&gt;59),1,_xlfn.XLOOKUP(E133,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="H133" s="3" t="str">
         <f>IF(G133="","",IF(G133="DNS",0,IF(G133="DQ",0,IF(G133="DNF",1,IF(AND(ISNUMBER(G133),G133&gt;59),1,_xlfn.XLOOKUP(G133,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -15265,18 +15261,18 @@
       </c>
       <c r="Q133" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="R133" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="S133" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="134" spans="1:19" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="134" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A134" t="s">
         <v>189</v>
       </c>
@@ -15806,25 +15802,25 @@
         <v>60</v>
       </c>
     </row>
-    <row r="144" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="144" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A144" t="s">
-        <v>186</v>
+        <v>359</v>
       </c>
       <c r="B144" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C144" t="s">
         <v>7</v>
       </c>
       <c r="D144" s="3">
-        <v>812</v>
+        <v>836</v>
       </c>
       <c r="E144" s="3">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="F144" s="3">
         <f>IF(E144="","",IF(E144="DNS",0,IF(E144="DQ",0,IF(E144="DNF",1,IF(AND(ISNUMBER(E144),E144&gt;59),1,_xlfn.XLOOKUP(E144,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="H144" s="3" t="str">
         <f>IF(G144="","",IF(G144="DNS",0,IF(G144="DQ",0,IF(G144="DNF",1,IF(AND(ISNUMBER(G144),G144&gt;59),1,_xlfn.XLOOKUP(G144,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -15848,15 +15844,15 @@
       </c>
       <c r="Q144" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="R144" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="S144" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>49</v>
+        <v>28</v>
       </c>
     </row>
     <row r="145" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -16124,25 +16120,25 @@
         <v>95</v>
       </c>
     </row>
-    <row r="150" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="150" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A150" t="s">
-        <v>185</v>
+        <v>103</v>
       </c>
       <c r="B150" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="C150" t="s">
         <v>7</v>
       </c>
       <c r="D150" s="3">
-        <v>811</v>
+        <v>8189</v>
       </c>
       <c r="E150" s="3">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="F150" s="3">
         <f>IF(E150="","",IF(E150="DNS",0,IF(E150="DQ",0,IF(E150="DNF",1,IF(AND(ISNUMBER(E150),E150&gt;59),1,_xlfn.XLOOKUP(E150,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="H150" s="3" t="str">
         <f>IF(G150="","",IF(G150="DNS",0,IF(G150="DQ",0,IF(G150="DNF",1,IF(AND(ISNUMBER(G150),G150&gt;59),1,_xlfn.XLOOKUP(G150,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -16166,15 +16162,15 @@
       </c>
       <c r="Q150" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="R150" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="S150" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>43</v>
+        <v>27</v>
       </c>
     </row>
     <row r="151" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -16230,9 +16226,9 @@
         <v>39</v>
       </c>
     </row>
-    <row r="152" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="152" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A152" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B152" t="s">
         <v>20</v>
@@ -16241,7 +16237,7 @@
         <v>7</v>
       </c>
       <c r="D152" s="3">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="E152" s="3">
         <v>34</v>
@@ -16283,7 +16279,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="153" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="153" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A153" t="s">
         <v>156</v>
       </c>
@@ -16336,7 +16332,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="154" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="154" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A154" t="s">
         <v>75</v>
       </c>
@@ -16389,7 +16385,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="155" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="155" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A155" t="s">
         <v>74</v>
       </c>
@@ -16442,7 +16438,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="156" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="156" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A156" t="s">
         <v>295</v>
       </c>
@@ -17025,25 +17021,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="167" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A167" t="s">
-        <v>183</v>
+        <v>332</v>
       </c>
       <c r="B167" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C167" t="s">
         <v>7</v>
       </c>
       <c r="D167" s="3">
-        <v>809</v>
-      </c>
-      <c r="E167" s="3" t="s">
-        <v>416</v>
+        <v>827</v>
+      </c>
+      <c r="E167" s="3">
+        <v>35</v>
       </c>
       <c r="F167" s="3">
         <f>IF(E167="","",IF(E167="DNS",0,IF(E167="DQ",0,IF(E167="DNF",1,IF(AND(ISNUMBER(E167),E167&gt;59),1,_xlfn.XLOOKUP(E167,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="H167" s="3" t="str">
         <f>IF(G167="","",IF(G167="DNS",0,IF(G167="DQ",0,IF(G167="DNF",1,IF(AND(ISNUMBER(G167),G167&gt;59),1,_xlfn.XLOOKUP(G167,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -17067,15 +17063,15 @@
       </c>
       <c r="Q167" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="R167" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="S167" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="168" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -18456,25 +18452,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="194" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A194" t="s">
-        <v>237</v>
+        <v>333</v>
       </c>
       <c r="B194" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C194" t="s">
         <v>7</v>
       </c>
       <c r="D194" s="3">
-        <v>814</v>
+        <v>828</v>
       </c>
       <c r="E194" s="3">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="F194" s="3">
         <f>IF(E194="","",IF(E194="DNS",0,IF(E194="DQ",0,IF(E194="DNF",1,IF(AND(ISNUMBER(E194),E194&gt;59),1,_xlfn.XLOOKUP(E194,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="H194" s="3" t="str">
         <f>IF(G194="","",IF(G194="DNS",0,IF(G194="DQ",0,IF(G194="DNF",1,IF(AND(ISNUMBER(G194),G194&gt;59),1,_xlfn.XLOOKUP(G194,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -18498,18 +18494,18 @@
       </c>
       <c r="Q194" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="R194" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="S194" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>42</v>
-      </c>
-    </row>
-    <row r="195" spans="1:19" x14ac:dyDescent="0.4">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="195" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A195" t="s">
         <v>124</v>
       </c>
@@ -18615,25 +18611,25 @@
         <v>1</v>
       </c>
     </row>
-    <row r="197" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="197" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A197" t="s">
-        <v>236</v>
+        <v>61</v>
       </c>
       <c r="B197" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="C197" t="s">
         <v>7</v>
       </c>
       <c r="D197" s="3">
-        <v>813</v>
+        <v>8185</v>
       </c>
       <c r="E197" s="3" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F197" s="3">
         <f>IF(E197="","",IF(E197="DNS",0,IF(E197="DQ",0,IF(E197="DNF",1,IF(AND(ISNUMBER(E197),E197&gt;59),1,_xlfn.XLOOKUP(E197,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H197" s="3" t="str">
         <f>IF(G197="","",IF(G197="DNS",0,IF(G197="DQ",0,IF(G197="DNF",1,IF(AND(ISNUMBER(G197),G197&gt;59),1,_xlfn.XLOOKUP(G197,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -18657,15 +18653,15 @@
       </c>
       <c r="Q197" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R197" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S197" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="198" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -18721,25 +18717,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="199" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A199" t="s">
-        <v>245</v>
+        <v>53</v>
       </c>
       <c r="B199" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="C199" t="s">
         <v>7</v>
       </c>
       <c r="D199" s="3">
-        <v>816</v>
-      </c>
-      <c r="E199" s="3">
-        <v>5</v>
+        <v>8010</v>
+      </c>
+      <c r="E199" s="3" t="s">
+        <v>416</v>
       </c>
       <c r="F199" s="3">
         <f>IF(E199="","",IF(E199="DNS",0,IF(E199="DQ",0,IF(E199="DNF",1,IF(AND(ISNUMBER(E199),E199&gt;59),1,_xlfn.XLOOKUP(E199,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="H199" s="3" t="str">
         <f>IF(G199="","",IF(G199="DNS",0,IF(G199="DQ",0,IF(G199="DNF",1,IF(AND(ISNUMBER(G199),G199&gt;59),1,_xlfn.XLOOKUP(G199,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -18763,15 +18759,15 @@
       </c>
       <c r="Q199" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="R199" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="S199" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>80</v>
+        <v>0</v>
       </c>
     </row>
     <row r="200" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -19092,25 +19088,25 @@
         <v>49</v>
       </c>
     </row>
-    <row r="206" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="206" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A206" t="s">
-        <v>246</v>
+        <v>55</v>
       </c>
       <c r="B206" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="C206" t="s">
         <v>7</v>
       </c>
       <c r="D206" s="3">
-        <v>817</v>
-      </c>
-      <c r="E206" s="3">
-        <v>14</v>
+        <v>8086</v>
+      </c>
+      <c r="E206" s="3" t="s">
+        <v>416</v>
       </c>
       <c r="F206" s="3">
         <f>IF(E206="","",IF(E206="DNS",0,IF(E206="DQ",0,IF(E206="DNF",1,IF(AND(ISNUMBER(E206),E206&gt;59),1,_xlfn.XLOOKUP(E206,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="H206" s="3" t="str">
         <f>IF(G206="","",IF(G206="DNS",0,IF(G206="DQ",0,IF(G206="DNF",1,IF(AND(ISNUMBER(G206),G206&gt;59),1,_xlfn.XLOOKUP(G206,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -19134,15 +19130,15 @@
       </c>
       <c r="Q206" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="R206" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="S206" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>47</v>
+        <v>0</v>
       </c>
     </row>
     <row r="207" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -19198,25 +19194,25 @@
         <v>36</v>
       </c>
     </row>
-    <row r="208" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="208" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A208" t="s">
-        <v>244</v>
+        <v>56</v>
       </c>
       <c r="B208" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="C208" t="s">
         <v>7</v>
       </c>
       <c r="D208" s="3">
-        <v>815</v>
-      </c>
-      <c r="E208" s="3">
-        <v>19</v>
+        <v>8140</v>
+      </c>
+      <c r="E208" s="3" t="s">
+        <v>416</v>
       </c>
       <c r="F208" s="3">
         <f>IF(E208="","",IF(E208="DNS",0,IF(E208="DQ",0,IF(E208="DNF",1,IF(AND(ISNUMBER(E208),E208&gt;59),1,_xlfn.XLOOKUP(E208,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="H208" s="3" t="str">
         <f>IF(G208="","",IF(G208="DNS",0,IF(G208="DQ",0,IF(G208="DNF",1,IF(AND(ISNUMBER(G208),G208&gt;59),1,_xlfn.XLOOKUP(G208,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -19240,15 +19236,15 @@
       </c>
       <c r="Q208" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="R208" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="S208" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="209" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -19993,7 +19989,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="223" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="223" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A223" t="s">
         <v>157</v>
       </c>
@@ -20046,7 +20042,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="224" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="224" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A224" t="s">
         <v>125</v>
       </c>
@@ -20099,7 +20095,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="225" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="225" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A225" t="s">
         <v>340</v>
       </c>
@@ -20152,7 +20148,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="226" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="226" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A226" t="s">
         <v>78</v>
       </c>
@@ -20205,7 +20201,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="227" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="227" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A227" t="s">
         <v>290</v>
       </c>
@@ -20788,25 +20784,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="238" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="238" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A238" t="s">
-        <v>281</v>
+        <v>58</v>
       </c>
       <c r="B238" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="C238" t="s">
         <v>7</v>
       </c>
       <c r="D238" s="3">
-        <v>819</v>
-      </c>
-      <c r="E238" s="3">
-        <v>28</v>
+        <v>8154</v>
+      </c>
+      <c r="E238" s="3" t="s">
+        <v>416</v>
       </c>
       <c r="F238" s="3">
         <f>IF(E238="","",IF(E238="DNS",0,IF(E238="DQ",0,IF(E238="DNF",1,IF(AND(ISNUMBER(E238),E238&gt;59),1,_xlfn.XLOOKUP(E238,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="H238" s="3" t="str">
         <f>IF(G238="","",IF(G238="DNS",0,IF(G238="DQ",0,IF(G238="DNF",1,IF(AND(ISNUMBER(G238),G238&gt;59),1,_xlfn.XLOOKUP(G238,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -20830,36 +20826,36 @@
       </c>
       <c r="Q238" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="R238" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="S238" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>32</v>
-      </c>
-    </row>
-    <row r="239" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="239" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A239" t="s">
-        <v>280</v>
+        <v>59</v>
       </c>
       <c r="B239" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="C239" t="s">
         <v>7</v>
       </c>
       <c r="D239" s="3">
-        <v>818</v>
-      </c>
-      <c r="E239" s="3">
-        <v>30</v>
+        <v>8177</v>
+      </c>
+      <c r="E239" s="3" t="s">
+        <v>416</v>
       </c>
       <c r="F239" s="3">
         <f>IF(E239="","",IF(E239="DNS",0,IF(E239="DQ",0,IF(E239="DNF",1,IF(AND(ISNUMBER(E239),E239&gt;59),1,_xlfn.XLOOKUP(E239,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="H239" s="3" t="str">
         <f>IF(G239="","",IF(G239="DNS",0,IF(G239="DQ",0,IF(G239="DNF",1,IF(AND(ISNUMBER(G239),G239&gt;59),1,_xlfn.XLOOKUP(G239,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -20883,15 +20879,15 @@
       </c>
       <c r="Q239" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="R239" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="S239" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>30</v>
+        <v>0</v>
       </c>
     </row>
     <row r="240" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -21477,7 +21473,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="251" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="251" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A251" t="s">
         <v>307</v>
       </c>
@@ -21530,7 +21526,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="252" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="252" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A252" t="s">
         <v>288</v>
       </c>
@@ -21583,7 +21579,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="253" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="253" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A253" t="s">
         <v>386</v>
       </c>
@@ -21636,7 +21632,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="254" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="254" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A254" t="s">
         <v>417</v>
       </c>
@@ -21689,7 +21685,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="255" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="255" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A255" t="s">
         <v>68</v>
       </c>
@@ -21742,7 +21738,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="256" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="256" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A256" t="s">
         <v>76</v>
       </c>
@@ -21795,7 +21791,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="257" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="257" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A257" t="s">
         <v>105</v>
       </c>
@@ -21848,7 +21844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="258" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="258" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A258" t="s">
         <v>166</v>
       </c>
@@ -21901,7 +21897,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="259" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="259" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A259" t="s">
         <v>167</v>
       </c>
@@ -21954,7 +21950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="260" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="260" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A260" t="s">
         <v>168</v>
       </c>
@@ -22007,7 +22003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="261" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="261" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A261" t="s">
         <v>169</v>
       </c>
@@ -22060,25 +22056,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="262" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="262" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A262" t="s">
-        <v>305</v>
+        <v>60</v>
       </c>
       <c r="B262" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="C262" t="s">
         <v>7</v>
       </c>
       <c r="D262" s="3">
-        <v>823</v>
-      </c>
-      <c r="E262" s="3">
-        <v>12</v>
+        <v>8181</v>
+      </c>
+      <c r="E262" s="3" t="s">
+        <v>416</v>
       </c>
       <c r="F262" s="3">
         <f>IF(E262="","",IF(E262="DNS",0,IF(E262="DQ",0,IF(E262="DNF",1,IF(AND(ISNUMBER(E262),E262&gt;59),1,_xlfn.XLOOKUP(E262,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="H262" s="3" t="str">
         <f>IF(G262="","",IF(G262="DNS",0,IF(G262="DQ",0,IF(G262="DNF",1,IF(AND(ISNUMBER(G262),G262&gt;59),1,_xlfn.XLOOKUP(G262,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -22102,15 +22098,15 @@
       </c>
       <c r="Q262" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="R262" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="S262" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>51</v>
+        <v>0</v>
       </c>
     </row>
     <row r="263" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -22166,25 +22162,25 @@
         <v>51</v>
       </c>
     </row>
-    <row r="264" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="264" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A264" t="s">
-        <v>302</v>
+        <v>62</v>
       </c>
       <c r="B264" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="C264" t="s">
         <v>7</v>
       </c>
       <c r="D264" s="3">
-        <v>820</v>
-      </c>
-      <c r="E264" s="3">
-        <v>20</v>
+        <v>8186</v>
+      </c>
+      <c r="E264" s="3" t="s">
+        <v>416</v>
       </c>
       <c r="F264" s="3">
         <f>IF(E264="","",IF(E264="DNS",0,IF(E264="DQ",0,IF(E264="DNF",1,IF(AND(ISNUMBER(E264),E264&gt;59),1,_xlfn.XLOOKUP(E264,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="H264" s="3" t="str">
         <f>IF(G264="","",IF(G264="DNS",0,IF(G264="DQ",0,IF(G264="DNF",1,IF(AND(ISNUMBER(G264),G264&gt;59),1,_xlfn.XLOOKUP(G264,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -22208,36 +22204,36 @@
       </c>
       <c r="Q264" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="R264" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="S264" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>40</v>
-      </c>
-    </row>
-    <row r="265" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="265" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A265" t="s">
-        <v>303</v>
+        <v>104</v>
       </c>
       <c r="B265" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="C265" t="s">
         <v>7</v>
       </c>
       <c r="D265" s="3">
-        <v>821</v>
-      </c>
-      <c r="E265" s="3">
-        <v>24</v>
+        <v>8190</v>
+      </c>
+      <c r="E265" s="3" t="s">
+        <v>416</v>
       </c>
       <c r="F265" s="3">
         <f>IF(E265="","",IF(E265="DNS",0,IF(E265="DQ",0,IF(E265="DNF",1,IF(AND(ISNUMBER(E265),E265&gt;59),1,_xlfn.XLOOKUP(E265,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="H265" s="3" t="str">
         <f>IF(G265="","",IF(G265="DNS",0,IF(G265="DQ",0,IF(G265="DNF",1,IF(AND(ISNUMBER(G265),G265&gt;59),1,_xlfn.XLOOKUP(G265,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -22261,36 +22257,36 @@
       </c>
       <c r="Q265" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="R265" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="S265" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="266" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="266" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A266" t="s">
-        <v>304</v>
+        <v>122</v>
       </c>
       <c r="B266" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="C266" t="s">
         <v>7</v>
       </c>
       <c r="D266" s="3">
-        <v>822</v>
-      </c>
-      <c r="E266" s="3">
-        <v>27</v>
+        <v>8193</v>
+      </c>
+      <c r="E266" s="3" t="s">
+        <v>416</v>
       </c>
       <c r="F266" s="3">
         <f>IF(E266="","",IF(E266="DNS",0,IF(E266="DQ",0,IF(E266="DNF",1,IF(AND(ISNUMBER(E266),E266&gt;59),1,_xlfn.XLOOKUP(E266,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="H266" s="3" t="str">
         <f>IF(G266="","",IF(G266="DNS",0,IF(G266="DQ",0,IF(G266="DNF",1,IF(AND(ISNUMBER(G266),G266&gt;59),1,_xlfn.XLOOKUP(G266,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -22314,18 +22310,18 @@
       </c>
       <c r="Q266" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="R266" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="S266" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>33</v>
-      </c>
-    </row>
-    <row r="267" spans="1:19" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="267" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A267" t="s">
         <v>177</v>
       </c>
@@ -22378,7 +22374,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="268" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="268" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A268" t="s">
         <v>188</v>
       </c>
@@ -22643,25 +22639,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="273" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="273" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A273" t="s">
-        <v>313</v>
+        <v>123</v>
       </c>
       <c r="B273" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="C273" t="s">
         <v>7</v>
       </c>
       <c r="D273" s="3">
-        <v>824</v>
-      </c>
-      <c r="E273" s="3">
-        <v>10</v>
+        <v>8194</v>
+      </c>
+      <c r="E273" s="3" t="s">
+        <v>416</v>
       </c>
       <c r="F273" s="3">
         <f>IF(E273="","",IF(E273="DNS",0,IF(E273="DQ",0,IF(E273="DNF",1,IF(AND(ISNUMBER(E273),E273&gt;59),1,_xlfn.XLOOKUP(E273,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="H273" s="3" t="str">
         <f>IF(G273="","",IF(G273="DNS",0,IF(G273="DQ",0,IF(G273="DNF",1,IF(AND(ISNUMBER(G273),G273&gt;59),1,_xlfn.XLOOKUP(G273,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -22685,36 +22681,36 @@
       </c>
       <c r="Q273" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="R273" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="S273" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>55</v>
-      </c>
-    </row>
-    <row r="274" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="274" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A274" t="s">
-        <v>314</v>
+        <v>139</v>
       </c>
       <c r="B274" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="C274" t="s">
         <v>7</v>
       </c>
       <c r="D274" s="3">
-        <v>825</v>
-      </c>
-      <c r="E274" s="3">
-        <v>13</v>
+        <v>8195</v>
+      </c>
+      <c r="E274" s="3" t="s">
+        <v>416</v>
       </c>
       <c r="F274" s="3">
         <f>IF(E274="","",IF(E274="DNS",0,IF(E274="DQ",0,IF(E274="DNF",1,IF(AND(ISNUMBER(E274),E274&gt;59),1,_xlfn.XLOOKUP(E274,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="H274" s="3" t="str">
         <f>IF(G274="","",IF(G274="DNS",0,IF(G274="DQ",0,IF(G274="DNF",1,IF(AND(ISNUMBER(G274),G274&gt;59),1,_xlfn.XLOOKUP(G274,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -22738,15 +22734,15 @@
       </c>
       <c r="Q274" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="R274" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="S274" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>49</v>
+        <v>0</v>
       </c>
     </row>
     <row r="275" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -23120,7 +23116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="282" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="282" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A282" t="s">
         <v>251</v>
       </c>
@@ -23173,7 +23169,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="283" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="283" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A283" t="s">
         <v>252</v>
       </c>
@@ -23226,7 +23222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="284" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="284" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A284" t="s">
         <v>253</v>
       </c>
@@ -23279,7 +23275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="285" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="285" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A285" t="s">
         <v>254</v>
       </c>
@@ -23703,25 +23699,25 @@
         <v>39</v>
       </c>
     </row>
-    <row r="293" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="293" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A293" t="s">
-        <v>331</v>
+        <v>146</v>
       </c>
       <c r="B293" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="C293" t="s">
         <v>7</v>
       </c>
       <c r="D293" s="3">
-        <v>826</v>
-      </c>
-      <c r="E293" s="3">
-        <v>16</v>
+        <v>801</v>
+      </c>
+      <c r="E293" s="3" t="s">
+        <v>416</v>
       </c>
       <c r="F293" s="3">
         <f>IF(E293="","",IF(E293="DNS",0,IF(E293="DQ",0,IF(E293="DNF",1,IF(AND(ISNUMBER(E293),E293&gt;59),1,_xlfn.XLOOKUP(E293,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="H293" s="3" t="str">
         <f>IF(G293="","",IF(G293="DNS",0,IF(G293="DQ",0,IF(G293="DNF",1,IF(AND(ISNUMBER(G293),G293&gt;59),1,_xlfn.XLOOKUP(G293,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -23745,36 +23741,36 @@
       </c>
       <c r="Q293" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="R293" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="S293" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>44</v>
-      </c>
-    </row>
-    <row r="294" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="294" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A294" t="s">
-        <v>334</v>
+        <v>144</v>
       </c>
       <c r="B294" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="C294" t="s">
         <v>7</v>
       </c>
       <c r="D294" s="3">
-        <v>829</v>
-      </c>
-      <c r="E294" s="3">
-        <v>21</v>
+        <v>8199</v>
+      </c>
+      <c r="E294" s="3" t="s">
+        <v>416</v>
       </c>
       <c r="F294" s="3">
         <f>IF(E294="","",IF(E294="DNS",0,IF(E294="DQ",0,IF(E294="DNF",1,IF(AND(ISNUMBER(E294),E294&gt;59),1,_xlfn.XLOOKUP(E294,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="H294" s="3" t="str">
         <f>IF(G294="","",IF(G294="DNS",0,IF(G294="DQ",0,IF(G294="DNF",1,IF(AND(ISNUMBER(G294),G294&gt;59),1,_xlfn.XLOOKUP(G294,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -23798,15 +23794,15 @@
       </c>
       <c r="Q294" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="R294" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="S294" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>39</v>
+        <v>0</v>
       </c>
     </row>
     <row r="295" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -23915,25 +23911,25 @@
         <v>26</v>
       </c>
     </row>
-    <row r="297" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="297" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A297" t="s">
-        <v>332</v>
+        <v>154</v>
       </c>
       <c r="B297" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="C297" t="s">
         <v>7</v>
       </c>
       <c r="D297" s="3">
-        <v>827</v>
-      </c>
-      <c r="E297" s="3">
-        <v>35</v>
+        <v>803</v>
+      </c>
+      <c r="E297" s="3" t="s">
+        <v>416</v>
       </c>
       <c r="F297" s="3">
         <f>IF(E297="","",IF(E297="DNS",0,IF(E297="DQ",0,IF(E297="DNF",1,IF(AND(ISNUMBER(E297),E297&gt;59),1,_xlfn.XLOOKUP(E297,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="H297" s="3" t="str">
         <f>IF(G297="","",IF(G297="DNS",0,IF(G297="DQ",0,IF(G297="DNF",1,IF(AND(ISNUMBER(G297),G297&gt;59),1,_xlfn.XLOOKUP(G297,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -23957,36 +23953,36 @@
       </c>
       <c r="Q297" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="R297" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="S297" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>25</v>
-      </c>
-    </row>
-    <row r="298" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="298" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A298" t="s">
-        <v>333</v>
+        <v>172</v>
       </c>
       <c r="B298" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="C298" t="s">
         <v>7</v>
       </c>
       <c r="D298" s="3">
-        <v>828</v>
-      </c>
-      <c r="E298" s="3">
-        <v>36</v>
+        <v>806</v>
+      </c>
+      <c r="E298" s="3" t="s">
+        <v>416</v>
       </c>
       <c r="F298" s="3">
         <f>IF(E298="","",IF(E298="DNS",0,IF(E298="DQ",0,IF(E298="DNF",1,IF(AND(ISNUMBER(E298),E298&gt;59),1,_xlfn.XLOOKUP(E298,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="H298" s="3" t="str">
         <f>IF(G298="","",IF(G298="DNS",0,IF(G298="DQ",0,IF(G298="DNF",1,IF(AND(ISNUMBER(G298),G298&gt;59),1,_xlfn.XLOOKUP(G298,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -24010,18 +24006,18 @@
       </c>
       <c r="Q298" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="R298" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="S298" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>24</v>
-      </c>
-    </row>
-    <row r="299" spans="1:19" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="299" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A299" t="s">
         <v>287</v>
       </c>
@@ -24074,7 +24070,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="300" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="300" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A300" t="s">
         <v>289</v>
       </c>
@@ -24127,7 +24123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="301" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="301" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A301" t="s">
         <v>294</v>
       </c>
@@ -24180,7 +24176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="302" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="302" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A302" t="s">
         <v>306</v>
       </c>
@@ -24233,7 +24229,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="303" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="303" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A303" t="s">
         <v>317</v>
       </c>
@@ -24397,18 +24393,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="306" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="306" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A306" t="s">
-        <v>335</v>
+        <v>173</v>
       </c>
       <c r="B306" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="C306" t="s">
         <v>7</v>
       </c>
       <c r="D306" s="3">
-        <v>830</v>
+        <v>807</v>
       </c>
       <c r="E306" s="3" t="s">
         <v>416</v>
@@ -24662,25 +24658,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="311" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="311" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A311" t="s">
-        <v>351</v>
+        <v>174</v>
       </c>
       <c r="B311" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="C311" t="s">
         <v>7</v>
       </c>
       <c r="D311" s="3">
-        <v>831</v>
-      </c>
-      <c r="E311" s="3">
-        <v>6</v>
+        <v>808</v>
+      </c>
+      <c r="E311" s="3" t="s">
+        <v>416</v>
       </c>
       <c r="F311" s="3">
         <f>IF(E311="","",IF(E311="DNS",0,IF(E311="DQ",0,IF(E311="DNF",1,IF(AND(ISNUMBER(E311),E311&gt;59),1,_xlfn.XLOOKUP(E311,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="H311" s="3" t="str">
         <f>IF(G311="","",IF(G311="DNS",0,IF(G311="DQ",0,IF(G311="DNF",1,IF(AND(ISNUMBER(G311),G311&gt;59),1,_xlfn.XLOOKUP(G311,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -24704,36 +24700,36 @@
       </c>
       <c r="Q311" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="R311" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="S311" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>75</v>
-      </c>
-    </row>
-    <row r="312" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="312" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A312" t="s">
-        <v>352</v>
+        <v>185</v>
       </c>
       <c r="B312" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C312" t="s">
         <v>7</v>
       </c>
       <c r="D312" s="3">
-        <v>832</v>
-      </c>
-      <c r="E312" s="3">
-        <v>7</v>
+        <v>811</v>
+      </c>
+      <c r="E312" s="3" t="s">
+        <v>416</v>
       </c>
       <c r="F312" s="3">
         <f>IF(E312="","",IF(E312="DNS",0,IF(E312="DQ",0,IF(E312="DNF",1,IF(AND(ISNUMBER(E312),E312&gt;59),1,_xlfn.XLOOKUP(E312,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="H312" s="3" t="str">
         <f>IF(G312="","",IF(G312="DNS",0,IF(G312="DQ",0,IF(G312="DNF",1,IF(AND(ISNUMBER(G312),G312&gt;59),1,_xlfn.XLOOKUP(G312,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -24757,18 +24753,18 @@
       </c>
       <c r="Q312" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="R312" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="S312" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>70</v>
-      </c>
-    </row>
-    <row r="313" spans="1:19" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="313" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A313" t="s">
         <v>319</v>
       </c>
@@ -24821,7 +24817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="314" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="314" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A314" t="s">
         <v>320</v>
       </c>
@@ -25298,25 +25294,25 @@
         <v>80</v>
       </c>
     </row>
-    <row r="323" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="323" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A323" t="s">
-        <v>356</v>
+        <v>236</v>
       </c>
       <c r="B323" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="C323" t="s">
         <v>7</v>
       </c>
       <c r="D323" s="3">
-        <v>833</v>
-      </c>
-      <c r="E323" s="3">
-        <v>15</v>
+        <v>813</v>
+      </c>
+      <c r="E323" s="3" t="s">
+        <v>416</v>
       </c>
       <c r="F323" s="3">
         <f>IF(E323="","",IF(E323="DNS",0,IF(E323="DQ",0,IF(E323="DNF",1,IF(AND(ISNUMBER(E323),E323&gt;59),1,_xlfn.XLOOKUP(E323,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="H323" s="3" t="str">
         <f>IF(G323="","",IF(G323="DNS",0,IF(G323="DQ",0,IF(G323="DNF",1,IF(AND(ISNUMBER(G323),G323&gt;59),1,_xlfn.XLOOKUP(G323,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -25340,36 +25336,36 @@
       </c>
       <c r="Q323" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="R323" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="S323" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>45</v>
-      </c>
-    </row>
-    <row r="324" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="324" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A324" t="s">
-        <v>359</v>
+        <v>335</v>
       </c>
       <c r="B324" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C324" t="s">
         <v>7</v>
       </c>
       <c r="D324" s="3">
-        <v>836</v>
-      </c>
-      <c r="E324" s="3">
-        <v>32</v>
+        <v>830</v>
+      </c>
+      <c r="E324" s="3" t="s">
+        <v>416</v>
       </c>
       <c r="F324" s="3">
         <f>IF(E324="","",IF(E324="DNS",0,IF(E324="DQ",0,IF(E324="DNF",1,IF(AND(ISNUMBER(E324),E324&gt;59),1,_xlfn.XLOOKUP(E324,tbl_points[Place],tbl_points[Points],""))))))</f>
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="H324" s="3" t="str">
         <f>IF(G324="","",IF(G324="DNS",0,IF(G324="DQ",0,IF(G324="DNF",1,IF(AND(ISNUMBER(G324),G324&gt;59),1,_xlfn.XLOOKUP(G324,tbl_points[Place],tbl_points[Points],""))))))</f>
@@ -25393,15 +25389,15 @@
       </c>
       <c r="Q324" s="3">
         <f>SUM(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="R324" s="3">
         <f>MIN(tbl_individual[[#This Row],[R1 Pts]],tbl_individual[[#This Row],[R2 Pts]],tbl_individual[[#This Row],[R3 Pts]],tbl_individual[[#This Row],[R4 Pts]],tbl_individual[[#This Row],[R5 Pts]],tbl_individual[[#This Row],[R6 Pts]])</f>
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="S324" s="3">
         <f>tbl_individual[[#This Row],[Total]]</f>
-        <v>28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="325" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
@@ -25669,7 +25665,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="330" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="330" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A330" t="s">
         <v>357</v>
       </c>
@@ -26093,7 +26089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="338" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="338" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A338" t="s">
         <v>358</v>
       </c>
@@ -26623,7 +26619,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="348" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="348" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A348" t="s">
         <v>336</v>
       </c>
@@ -26676,7 +26672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="349" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="349" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A349" t="s">
         <v>384</v>
       </c>
@@ -26729,7 +26725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="350" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="350" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
       <c r="A350" t="s">
         <v>385</v>
       </c>
@@ -26835,7 +26831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="352" spans="1:19" hidden="1" x14ac:dyDescent="0.4">
+    <row r="352" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A352" t="s">
         <v>383</v>
       </c>
@@ -29411,7 +29407,7 @@
     ""
 )
 )</f>
-        <v>118</v>
+        <v>98</v>
       </c>
       <c r="D6" s="3" t="str" cm="1">
         <f t="array" ref="D6">_xlfn.LET(
@@ -29580,7 +29576,7 @@
       </c>
       <c r="I6" s="3">
         <f>SUM(tbl_teampoints[[#This Row],[Race 1]]:tbl_teampoints[[#This Row],[Race 6]])</f>
-        <v>118</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.4">
@@ -39785,16 +39781,16 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" t="str">
-        <v>Max Remfry</v>
+        <v>Kelyn Horsely</v>
       </c>
       <c r="B23" t="str">
-        <v>Argyle</v>
+        <v>Don Ross</v>
       </c>
       <c r="C23" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D23">
-        <v>8147</v>
+        <v>837</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.4">
@@ -39827,16 +39823,16 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A26" t="str">
-        <v>Laith Rifaat</v>
+        <v>Elias Newby</v>
       </c>
       <c r="B26" t="str">
-        <v>Argyle</v>
+        <v>Don Ross</v>
       </c>
       <c r="C26" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D26">
-        <v>8049</v>
+        <v>838</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.4">
@@ -39981,44 +39977,44 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A37" t="str">
-        <v>Owen Purdy</v>
+        <v>Alexander Moran</v>
       </c>
       <c r="B37" t="str">
-        <v>Argyle</v>
+        <v>Chatelech</v>
       </c>
       <c r="C37" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D37">
-        <v>8185</v>
+        <v>8196</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A38" t="str">
-        <v>Ryan Pasha</v>
+        <v>Asher Lissett</v>
       </c>
       <c r="B38" t="str">
-        <v>Argyle</v>
+        <v>Coast Mtn</v>
       </c>
       <c r="C38" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D38">
-        <v>8010</v>
+        <v>8198</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A39" t="str">
-        <v>Dylan MacDondald</v>
+        <v>Tristan Clark</v>
       </c>
       <c r="B39" t="str">
-        <v>Argyle</v>
+        <v>Don Ross</v>
       </c>
       <c r="C39" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D39">
-        <v>8086</v>
+        <v>839</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.4">
@@ -40177,72 +40173,72 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A51" t="str">
-        <v>Lucas Cullingworth</v>
+        <v>Dash Nicoll</v>
       </c>
       <c r="B51" t="str">
-        <v>Argyle</v>
+        <v>Pemberton</v>
       </c>
       <c r="C51" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D51">
-        <v>8140</v>
+        <v>816</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A52" t="str">
-        <v>Riley Buxton</v>
+        <v>Hayden Bristow</v>
       </c>
       <c r="B52" t="str">
-        <v>Argyle</v>
+        <v>West Van</v>
       </c>
       <c r="C52" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D52">
-        <v>8154</v>
+        <v>831</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A53" t="str">
-        <v>Rowen Doerr</v>
+        <v>Trent Bristow</v>
       </c>
       <c r="B53" t="str">
-        <v>Argyle</v>
+        <v>West Van</v>
       </c>
       <c r="C53" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D53">
-        <v>8177</v>
+        <v>832</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A54" t="str">
-        <v>Ronin Stewart</v>
+        <v>Slater McDougall</v>
       </c>
       <c r="B54" t="str">
-        <v>Argyle</v>
+        <v>Collingwood</v>
       </c>
       <c r="C54" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D54">
-        <v>8181</v>
+        <v>804</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A55" t="str">
-        <v>Nico Scott</v>
+        <v>Callum Paul</v>
       </c>
       <c r="B55" t="str">
-        <v>Argyle</v>
+        <v>Coast Mtn</v>
       </c>
       <c r="C55" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D55">
-        <v>8186</v>
+        <v>8009</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.4">
@@ -40303,16 +40299,16 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A60" t="str">
-        <v>Aiden Bucci</v>
+        <v>Teo Damici</v>
       </c>
       <c r="B60" t="str">
-        <v>Brockton</v>
+        <v>STA</v>
       </c>
       <c r="C60" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D60">
-        <v>8189</v>
+        <v>824</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.4">
@@ -40401,16 +40397,16 @@
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A67" t="str">
-        <v>Henry Sparrow</v>
+        <v>Andrew Simpson</v>
       </c>
       <c r="B67" t="str">
-        <v>Brockton</v>
+        <v>Coast Mtn</v>
       </c>
       <c r="C67" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D67">
-        <v>8190</v>
+        <v>8197</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.4">
@@ -40429,30 +40425,30 @@
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A69" t="str">
-        <v>Austin Bandic</v>
+        <v>Andrew Wenzlaff</v>
       </c>
       <c r="B69" t="str">
-        <v>Burnaby Mtn</v>
+        <v>St. Georges</v>
       </c>
       <c r="C69" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D69">
-        <v>8191</v>
+        <v>823</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A70" t="str">
-        <v>Yara Raouf Malayeri</v>
+        <v>Rory Sykes</v>
       </c>
       <c r="B70" t="str">
-        <v>Burnaby Mtn</v>
+        <v>STA</v>
       </c>
       <c r="C70" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D70">
-        <v>8192</v>
+        <v>825</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.4">
@@ -40726,30 +40722,30 @@
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A90" t="str">
-        <v>James Kwong</v>
+        <v>Micah Treadway</v>
       </c>
       <c r="B90" t="str">
-        <v>Carson</v>
+        <v>Pemberton</v>
       </c>
       <c r="C90" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D90">
-        <v>8193</v>
+        <v>817</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A91" t="str">
-        <v>Bryce Weatherly</v>
+        <v>Luke McGowan</v>
       </c>
       <c r="B91" t="str">
-        <v>Carson</v>
+        <v>Whistler</v>
       </c>
       <c r="C91" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D91">
-        <v>8194</v>
+        <v>833</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.4">
@@ -40782,16 +40778,16 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A94" t="str">
-        <v>Alexander Moran</v>
+        <v>William Kolper</v>
       </c>
       <c r="B94" t="str">
-        <v>Chatelech</v>
+        <v>Sutherland</v>
       </c>
       <c r="C94" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D94">
-        <v>8196</v>
+        <v>826</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.4">
@@ -40824,30 +40820,30 @@
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A97" t="str">
-        <v>Jack Walton</v>
+        <v>Felix Carr</v>
       </c>
       <c r="B97" t="str">
-        <v>Chatelech</v>
+        <v>Handsworth</v>
       </c>
       <c r="C97" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D97">
-        <v>8195</v>
+        <v>810</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A98" t="str">
-        <v>Asher Lissett</v>
+        <v>Lennart Schilling</v>
       </c>
       <c r="B98" t="str">
-        <v>Coast Mtn</v>
+        <v>Mulgrave</v>
       </c>
       <c r="C98" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D98">
-        <v>8198</v>
+        <v>814</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.4">
@@ -40866,30 +40862,30 @@
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A100" t="str">
-        <v>Callum Paul</v>
+        <v>Ryan Kearnes</v>
       </c>
       <c r="B100" t="str">
-        <v>Coast Mtn</v>
+        <v>Pemberton</v>
       </c>
       <c r="C100" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D100">
-        <v>8009</v>
+        <v>815</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A101" t="str">
-        <v>Andrew Simpson</v>
+        <v>Tristan Cole</v>
       </c>
       <c r="B101" t="str">
-        <v>Coast Mtn</v>
+        <v>St. Georges</v>
       </c>
       <c r="C101" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D101">
-        <v>8197</v>
+        <v>820</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.4">
@@ -40908,16 +40904,16 @@
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A103" t="str">
-        <v>Jackson Jones</v>
+        <v>Seth Andru</v>
       </c>
       <c r="B103" t="str">
-        <v>Coast Mtn</v>
+        <v>Sutherland</v>
       </c>
       <c r="C103" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D103">
-        <v>800</v>
+        <v>829</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.4">
@@ -40978,44 +40974,44 @@
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A108" t="str">
-        <v>Cole Fraser</v>
+        <v>Austin Bandic</v>
       </c>
       <c r="B108" t="str">
-        <v>Coast Mtn</v>
+        <v>Burnaby Mtn</v>
       </c>
       <c r="C108" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D108">
-        <v>801</v>
+        <v>8191</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A109" t="str">
-        <v>Weston Morum</v>
+        <v>Max Remfry</v>
       </c>
       <c r="B109" t="str">
-        <v>Coast Mtn</v>
+        <v>Argyle</v>
       </c>
       <c r="C109" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D109">
-        <v>8199</v>
+        <v>8147</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A110" t="str">
-        <v>Slater McDougall</v>
+        <v>Alasdair Robertson</v>
       </c>
       <c r="B110" t="str">
-        <v>Collingwood</v>
+        <v>St. Georges</v>
       </c>
       <c r="C110" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D110">
-        <v>804</v>
+        <v>821</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.4">
@@ -41118,58 +41114,58 @@
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A118" t="str">
-        <v>Jack Burt</v>
+        <v>Laith Rifaat</v>
       </c>
       <c r="B118" t="str">
-        <v>Collingwood</v>
+        <v>Argyle</v>
       </c>
       <c r="C118" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D118">
-        <v>803</v>
+        <v>8049</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A119" t="str">
-        <v>Kelyn Horsely</v>
+        <v>Jackson Jones</v>
       </c>
       <c r="B119" t="str">
-        <v>Don Ross</v>
+        <v>Coast Mtn</v>
       </c>
       <c r="C119" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D119">
-        <v>837</v>
+        <v>800</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A120" t="str">
-        <v>Elias Newby</v>
+        <v>David Shilletto</v>
       </c>
       <c r="B120" t="str">
-        <v>Don Ross</v>
+        <v>St. Georges</v>
       </c>
       <c r="C120" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D120">
-        <v>838</v>
+        <v>822</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A121" t="str">
-        <v>Tristan Clark</v>
+        <v>Augusten Worsfold</v>
       </c>
       <c r="B121" t="str">
-        <v>Don Ross</v>
+        <v>Rockridge</v>
       </c>
       <c r="C121" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D121">
-        <v>839</v>
+        <v>819</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.4">
@@ -41272,16 +41268,16 @@
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A129" t="str">
-        <v>Jivcko Elvir Sheilds</v>
+        <v>Yara Raouf Malayeri</v>
       </c>
       <c r="B129" t="str">
-        <v>Elphinstone</v>
+        <v>Burnaby Mtn</v>
       </c>
       <c r="C129" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D129">
-        <v>806</v>
+        <v>8192</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.4">
@@ -41314,16 +41310,16 @@
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A132" t="str">
-        <v>Sean Weber</v>
+        <v>Lucas Solis</v>
       </c>
       <c r="B132" t="str">
-        <v>Elphinstone</v>
+        <v>Rockridge</v>
       </c>
       <c r="C132" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D132">
-        <v>807</v>
+        <v>818</v>
       </c>
       <c r="E132" s="3" t="s">
         <v>412</v>
@@ -41331,16 +41327,16 @@
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A133" t="str">
-        <v>Arthur Scale</v>
+        <v>Remy Zurbuchen</v>
       </c>
       <c r="B133" t="str">
-        <v>Elphinstone</v>
+        <v>Handsworth</v>
       </c>
       <c r="C133" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D133">
-        <v>808</v>
+        <v>812</v>
       </c>
       <c r="E133" s="3" t="s">
         <v>412</v>
@@ -41500,16 +41496,16 @@
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A144" t="str">
-        <v>Remy Zurbuchen</v>
+        <v>Anton Anghellescu</v>
       </c>
       <c r="B144" t="str">
-        <v>Handsworth</v>
+        <v>Whistler</v>
       </c>
       <c r="C144" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D144">
-        <v>812</v>
+        <v>836</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.4">
@@ -41584,16 +41580,16 @@
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A150" t="str">
-        <v>William Lucas</v>
+        <v>Aiden Bucci</v>
       </c>
       <c r="B150" t="str">
-        <v>Handsworth</v>
+        <v>Brockton</v>
       </c>
       <c r="C150" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D150">
-        <v>811</v>
+        <v>8189</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.4">
@@ -41612,7 +41608,7 @@
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A152" t="str">
-        <v>Felix Carr</v>
+        <v>Marcelo Alcocer Tremari</v>
       </c>
       <c r="B152" t="str">
         <v>Handsworth</v>
@@ -41621,7 +41617,7 @@
         <v>Bant Boys</v>
       </c>
       <c r="D152">
-        <v>810</v>
+        <v>809</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.4">
@@ -41822,16 +41818,16 @@
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A167" t="str">
-        <v>Marcelo Alcocer Tremari</v>
+        <v>Erik Moore</v>
       </c>
       <c r="B167" t="str">
-        <v>Handsworth</v>
+        <v>Sutherland</v>
       </c>
       <c r="C167" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D167">
-        <v>809</v>
+        <v>827</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.4">
@@ -42200,16 +42196,16 @@
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A194" t="str">
-        <v>Lennart Schilling</v>
+        <v>Kaelan Percival</v>
       </c>
       <c r="B194" t="str">
-        <v>Mulgrave</v>
+        <v>Sutherland</v>
       </c>
       <c r="C194" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D194">
-        <v>814</v>
+        <v>828</v>
       </c>
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.4">
@@ -42242,16 +42238,16 @@
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A197" t="str">
-        <v>Jeronimo Gomez</v>
+        <v>Owen Purdy</v>
       </c>
       <c r="B197" t="str">
-        <v>Mulgrave</v>
+        <v>Argyle</v>
       </c>
       <c r="C197" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D197">
-        <v>813</v>
+        <v>8185</v>
       </c>
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.4">
@@ -42270,16 +42266,16 @@
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A199" t="str">
-        <v>Dash Nicoll</v>
+        <v>Ryan Pasha</v>
       </c>
       <c r="B199" t="str">
-        <v>Pemberton</v>
+        <v>Argyle</v>
       </c>
       <c r="C199" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D199">
-        <v>816</v>
+        <v>8010</v>
       </c>
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.4">
@@ -42368,16 +42364,16 @@
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A206" t="str">
-        <v>Micah Treadway</v>
+        <v>Dylan MacDondald</v>
       </c>
       <c r="B206" t="str">
-        <v>Pemberton</v>
+        <v>Argyle</v>
       </c>
       <c r="C206" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D206">
-        <v>817</v>
+        <v>8086</v>
       </c>
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.4">
@@ -42396,16 +42392,16 @@
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A208" t="str">
-        <v>Ryan Kearnes</v>
+        <v>Lucas Cullingworth</v>
       </c>
       <c r="B208" t="str">
-        <v>Pemberton</v>
+        <v>Argyle</v>
       </c>
       <c r="C208" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D208">
-        <v>815</v>
+        <v>8140</v>
       </c>
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.4">
@@ -42816,30 +42812,30 @@
     </row>
     <row r="238" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A238" t="str">
-        <v>Augusten Worsfold</v>
+        <v>Riley Buxton</v>
       </c>
       <c r="B238" t="str">
-        <v>Rockridge</v>
+        <v>Argyle</v>
       </c>
       <c r="C238" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D238">
-        <v>819</v>
+        <v>8154</v>
       </c>
     </row>
     <row r="239" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A239" t="str">
-        <v>Lucas Solis</v>
+        <v>Rowen Doerr</v>
       </c>
       <c r="B239" t="str">
-        <v>Rockridge</v>
+        <v>Argyle</v>
       </c>
       <c r="C239" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D239">
-        <v>818</v>
+        <v>8177</v>
       </c>
     </row>
     <row r="240" spans="1:4" x14ac:dyDescent="0.4">
@@ -43164,16 +43160,16 @@
     </row>
     <row r="262" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A262" t="str">
-        <v>Andrew Wenzlaff</v>
+        <v>Ronin Stewart</v>
       </c>
       <c r="B262" t="str">
-        <v>St. Georges</v>
+        <v>Argyle</v>
       </c>
       <c r="C262" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D262">
-        <v>823</v>
+        <v>8181</v>
       </c>
       <c r="E262" s="3" t="s">
         <v>407</v>
@@ -43198,16 +43194,16 @@
     </row>
     <row r="264" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A264" t="str">
-        <v>Tristan Cole</v>
+        <v>Nico Scott</v>
       </c>
       <c r="B264" t="str">
-        <v>St. Georges</v>
+        <v>Argyle</v>
       </c>
       <c r="C264" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D264">
-        <v>820</v>
+        <v>8186</v>
       </c>
       <c r="E264" s="3" t="s">
         <v>407</v>
@@ -43215,16 +43211,16 @@
     </row>
     <row r="265" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A265" t="str">
-        <v>Alasdair Robertson</v>
+        <v>Henry Sparrow</v>
       </c>
       <c r="B265" t="str">
-        <v>St. Georges</v>
+        <v>Brockton</v>
       </c>
       <c r="C265" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D265">
-        <v>821</v>
+        <v>8190</v>
       </c>
       <c r="E265" s="3" t="s">
         <v>407</v>
@@ -43232,16 +43228,16 @@
     </row>
     <row r="266" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A266" t="str">
-        <v>David Shilletto</v>
+        <v>James Kwong</v>
       </c>
       <c r="B266" t="str">
-        <v>St. Georges</v>
+        <v>Carson</v>
       </c>
       <c r="C266" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D266">
-        <v>822</v>
+        <v>8193</v>
       </c>
       <c r="E266" s="3" t="s">
         <v>407</v>
@@ -43339,30 +43335,30 @@
     </row>
     <row r="273" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A273" t="str">
-        <v>Teo Damici</v>
+        <v>Bryce Weatherly</v>
       </c>
       <c r="B273" t="str">
-        <v>STA</v>
+        <v>Carson</v>
       </c>
       <c r="C273" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D273">
-        <v>824</v>
+        <v>8194</v>
       </c>
     </row>
     <row r="274" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A274" t="str">
-        <v>Rory Sykes</v>
+        <v>Jack Walton</v>
       </c>
       <c r="B274" t="str">
-        <v>STA</v>
+        <v>Chatelech</v>
       </c>
       <c r="C274" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D274">
-        <v>825</v>
+        <v>8195</v>
       </c>
     </row>
     <row r="275" spans="1:4" x14ac:dyDescent="0.4">
@@ -43625,30 +43621,30 @@
     </row>
     <row r="293" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A293" t="str">
-        <v>William Kolper</v>
+        <v>Cole Fraser</v>
       </c>
       <c r="B293" t="str">
-        <v>Sutherland</v>
+        <v>Coast Mtn</v>
       </c>
       <c r="C293" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D293">
-        <v>826</v>
+        <v>801</v>
       </c>
     </row>
     <row r="294" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A294" t="str">
-        <v>Seth Andru</v>
+        <v>Weston Morum</v>
       </c>
       <c r="B294" t="str">
-        <v>Sutherland</v>
+        <v>Coast Mtn</v>
       </c>
       <c r="C294" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D294">
-        <v>829</v>
+        <v>8199</v>
       </c>
     </row>
     <row r="295" spans="1:5" x14ac:dyDescent="0.4">
@@ -43681,30 +43677,30 @@
     </row>
     <row r="297" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A297" t="str">
-        <v>Erik Moore</v>
+        <v>Jack Burt</v>
       </c>
       <c r="B297" t="str">
-        <v>Sutherland</v>
+        <v>Collingwood</v>
       </c>
       <c r="C297" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D297">
-        <v>827</v>
+        <v>803</v>
       </c>
     </row>
     <row r="298" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A298" t="str">
-        <v>Kaelan Percival</v>
+        <v>Jivcko Elvir Sheilds</v>
       </c>
       <c r="B298" t="str">
-        <v>Sutherland</v>
+        <v>Elphinstone</v>
       </c>
       <c r="C298" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D298">
-        <v>828</v>
+        <v>806</v>
       </c>
     </row>
     <row r="299" spans="1:5" x14ac:dyDescent="0.4">
@@ -43807,16 +43803,16 @@
     </row>
     <row r="306" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A306" t="str">
-        <v>Greyson Klein</v>
+        <v>Sean Weber</v>
       </c>
       <c r="B306" t="str">
-        <v>Sutherland</v>
+        <v>Elphinstone</v>
       </c>
       <c r="C306" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D306">
-        <v>830</v>
+        <v>807</v>
       </c>
     </row>
     <row r="307" spans="1:4" x14ac:dyDescent="0.4">
@@ -43877,30 +43873,30 @@
     </row>
     <row r="311" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A311" t="str">
-        <v>Hayden Bristow</v>
+        <v>Arthur Scale</v>
       </c>
       <c r="B311" t="str">
-        <v>West Van</v>
+        <v>Elphinstone</v>
       </c>
       <c r="C311" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D311">
-        <v>831</v>
+        <v>808</v>
       </c>
     </row>
     <row r="312" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A312" t="str">
-        <v>Trent Bristow</v>
+        <v>William Lucas</v>
       </c>
       <c r="B312" t="str">
-        <v>West Van</v>
+        <v>Handsworth</v>
       </c>
       <c r="C312" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D312">
-        <v>832</v>
+        <v>811</v>
       </c>
     </row>
     <row r="313" spans="1:4" x14ac:dyDescent="0.4">
@@ -44045,30 +44041,30 @@
     </row>
     <row r="323" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A323" t="str">
-        <v>Luke McGowan</v>
+        <v>Jeronimo Gomez</v>
       </c>
       <c r="B323" t="str">
-        <v>Whistler</v>
+        <v>Mulgrave</v>
       </c>
       <c r="C323" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D323">
-        <v>833</v>
+        <v>813</v>
       </c>
     </row>
     <row r="324" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A324" t="str">
-        <v>Anton Anghellescu</v>
+        <v>Greyson Klein</v>
       </c>
       <c r="B324" t="str">
-        <v>Whistler</v>
+        <v>Sutherland</v>
       </c>
       <c r="C324" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D324">
-        <v>836</v>
+        <v>830</v>
       </c>
     </row>
     <row r="325" spans="1:4" x14ac:dyDescent="0.4">
@@ -44579,16 +44575,16 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A6" t="str">
-        <v>Andrew Wenzlaff</v>
+        <v>Ronin Stewart</v>
       </c>
       <c r="B6" t="str">
-        <v>St. Georges</v>
+        <v>Argyle</v>
       </c>
       <c r="C6" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D6">
-        <v>823</v>
+        <v>8181</v>
       </c>
       <c r="E6" s="3" t="str">
         <v>yes</v>
@@ -44613,16 +44609,16 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A8" t="str">
-        <v>Tristan Cole</v>
+        <v>Nico Scott</v>
       </c>
       <c r="B8" t="str">
-        <v>St. Georges</v>
+        <v>Argyle</v>
       </c>
       <c r="C8" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D8">
-        <v>820</v>
+        <v>8186</v>
       </c>
       <c r="E8" s="3" t="str">
         <v>yes</v>
@@ -44630,16 +44626,16 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A9" t="str">
-        <v>Alasdair Robertson</v>
+        <v>Henry Sparrow</v>
       </c>
       <c r="B9" t="str">
-        <v>St. Georges</v>
+        <v>Brockton</v>
       </c>
       <c r="C9" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D9">
-        <v>821</v>
+        <v>8190</v>
       </c>
       <c r="E9" s="3" t="str">
         <v>yes</v>
@@ -44647,16 +44643,16 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A10" t="str">
-        <v>David Shilletto</v>
+        <v>James Kwong</v>
       </c>
       <c r="B10" t="str">
-        <v>St. Georges</v>
+        <v>Carson</v>
       </c>
       <c r="C10" t="str">
         <v>Bant Boys</v>
       </c>
       <c r="D10">
-        <v>822</v>
+        <v>8193</v>
       </c>
       <c r="E10" s="3" t="str">
         <v>yes</v>

</xml_diff>